<commit_message>
provided feedback bach#2 images
</commit_message>
<xml_diff>
--- a/outputs/session_log.xlsx
+++ b/outputs/session_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ramakant\VSCode-projects\delicut-creative-workflow\outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{915BA5EF-3403-4BE7-BFAD-67E70AD11B98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85FAEFAC-4CE3-4561-8458-85B3DFAF4C81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="53">
   <si>
     <t>session_id</t>
   </si>
@@ -79,6 +79,9 @@
     <t>ERROR: 404 NOT_FOUND. {'error': {'code': 404, 'message': 'models\imagen-3.0-generate-002 is not found for API version v1beta, or is not supported for predict. Call ListModels to see the list of available models and their supported methods.', 'status': 'NOT_FOUND'}}</t>
   </si>
   <si>
+    <t>reject</t>
+  </si>
+  <si>
     <t>B</t>
   </si>
   <si>
@@ -115,31 +118,70 @@
     <t>outputs\images\harry_0317-1502_locker-room-male_Imagen4Ultra.png</t>
   </si>
   <si>
+    <t xml:space="preserve">image generation is below par. Not in line with the our internal standards. </t>
+  </si>
+  <si>
     <t>outputs\images\harry_0317-1502_hands-contrast_Imagen4Ultra.png</t>
   </si>
   <si>
+    <t>delicut meal box has not been used. How do we consider references from the top performing images provided? Also the hands are generated in a weird way as though they are different hands</t>
+  </si>
+  <si>
     <t>outputs\images\harry_0317-1502_treadmill-female_Imagen4Ultra.png</t>
   </si>
   <si>
+    <t>seems alright. Needs modification and alternatives</t>
+  </si>
+  <si>
+    <t>to refine</t>
+  </si>
+  <si>
     <t>outputs\images\harry_0317-1502_abstract-green_Imagen4Ultra.png</t>
   </si>
   <si>
-    <t xml:space="preserve">image generation is below par. Not in line with the our internal standards. </t>
-  </si>
-  <si>
-    <t>reject</t>
-  </si>
-  <si>
-    <t>delicut meal box has not been used. How do we consider references from the top performing images provided? Also the hands are generated in a weird way as though they are different hands</t>
-  </si>
-  <si>
-    <t>seems alright. Needs modification and alternatives</t>
-  </si>
-  <si>
-    <t>to refine</t>
-  </si>
-  <si>
     <t xml:space="preserve">reject because no product images have been generated. How to use the delicut meal boxes as shown in the top performing creatives folder? </t>
+  </si>
+  <si>
+    <t>harry_0317-1622</t>
+  </si>
+  <si>
+    <t>Athletic male, 28–32, lean defined physique, sitting alone on a wooden gym locker room bench post-workout. Wearing dark fitted compression shorts and a sleeveless training top. Forearms resting on knees, head slightly down, composed and focused expression. Natural side light from a high window casting soft shadows across the locker room. A 900ml square meal prep tray with soft rounded corners, warm beige matte base and clear rigid plastic lid with a bold red label band reading '/delicut/' sits on the bench beside his gym bag. Shallow depth of field, locker room softly blurred in background. No other text. No other branding. Photorealistic, cinematic, shot on 35mm, muted warm tones. 1080x1080.</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0317-1622_locker-room-male_Imagen4Ultra.png</t>
+  </si>
+  <si>
+    <t>Close-up of a single pair of athletic male hands on a dark gym floor. Left hand grips a clear protein shaker, right hand rests beside a 900ml square meal prep tray with warm beige base and clear lid with a bold red '/delicut/' label band. Both objects on the same surface, hands natural and relaxed. Single overhead studio light, deep clean shadows. No face visible. No other text. No other branding. Photorealistic, commercial photography, high contrast, sharp focus. 1080x1080.</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0317-1622_hands-contrast_Imagen4Ultra.png</t>
+  </si>
+  <si>
+    <t>Lean athletic female, mid-20s, running powerfully on a treadmill in a bright modern gym. Wearing a fitted sports bra and high-waist shorts with midriff visible. Hair tied back in a high ponytail, strong forward gaze, confident expression. Legs in mid-stride, slight motion blur suggesting speed. Bright overhead gym lighting, mirrors and equipment softly visible in background. Shot from a slight front-side angle at eye level. Natural athletic proportions, strong posture. No text. No branding. No logos. Photorealistic, energetic, shot on 50mm, bright and clean. 1080x1080.</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0317-1622_treadmill-female_Imagen4Ultra.png</t>
+  </si>
+  <si>
+    <t>Top-down flat-lay on a deep spinach green surface, hex #043F12. Centre frame: a 900ml square meal prep tray with warm beige matte base, clear rigid plastic lid, bold red wraparound label band reading '/delicut/' in white. Arranged around it: a single white chalk-dusted weight plate, a neatly folded white gym towel, a stainless steel water bottle. Hard studio overhead lighting, crisp clean shadows, generous negative space. No additional text. No other branding. Commercial product photography, ultra-clean, high resolution. 1080x1080.</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0317-1622_abstract-green_Imagen4Ultra.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reject. Delicut product image and human features are not as per satisfaction. Ad copy doesn't seem to inherting or inspired from this image. </t>
+  </si>
+  <si>
+    <t>delicut meal box is empty without food which makes this very unlikely. Protein shaker is not placed properly</t>
+  </si>
+  <si>
+    <t>only concept that seems working</t>
+  </si>
+  <si>
+    <t>this might work. But needs appropriate ad copy</t>
+  </si>
+  <si>
+    <t>approved</t>
   </si>
 </sst>
 </file>
@@ -496,7 +538,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="11" width="22" customWidth="1"/>
@@ -537,7 +579,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="331.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="331.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
@@ -565,10 +607,10 @@
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="288" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="288" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
@@ -579,7 +621,7 @@
         <v>1</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>14</v>
@@ -588,7 +630,7 @@
         <v>15</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>17</v>
@@ -596,10 +638,10 @@
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
       <c r="K3" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="331.2" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="331.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -610,7 +652,7 @@
         <v>1</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>14</v>
@@ -619,7 +661,7 @@
         <v>15</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>17</v>
@@ -627,10 +669,10 @@
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="316.8" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="316.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
@@ -641,7 +683,7 @@
         <v>1</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>14</v>
@@ -650,7 +692,7 @@
         <v>15</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>17</v>
@@ -658,12 +700,12 @@
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="331.2" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="331.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>12</v>
@@ -675,7 +717,7 @@
         <v>13</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>15</v>
@@ -684,17 +726,17 @@
         <v>16</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
       <c r="K6" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="288" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="288" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>12</v>
@@ -703,29 +745,29 @@
         <v>1</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
       <c r="K7" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="331.2" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="331.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>12</v>
@@ -734,60 +776,60 @@
         <v>1</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>15</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="316.8" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="316.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="2">
+        <v>1</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="2">
-        <v>1</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>23</v>
-      </c>
       <c r="H9" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
       <c r="K9" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="331.2" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="331.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>12</v>
@@ -799,7 +841,7 @@
         <v>13</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>15</v>
@@ -808,112 +850,112 @@
         <v>16</v>
       </c>
       <c r="H10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10" s="2">
+        <v>1</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="288" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="2">
+        <v>1</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="I10" s="2">
-        <v>1</v>
-      </c>
-      <c r="J10" s="2" t="s">
+      <c r="F11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I11" s="2">
+        <v>1</v>
+      </c>
+      <c r="J11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K10" s="2" t="s">
+      <c r="K11" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="331.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="2">
+        <v>1</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H12" s="2" t="s">
         <v>34</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="288" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" s="2">
-        <v>1</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="I11" s="2">
-        <v>1</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="K11" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="331.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" s="2">
-        <v>1</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>31</v>
       </c>
       <c r="I12" s="2">
         <v>3</v>
       </c>
       <c r="J12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K12" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="K12" s="2" t="s">
+    </row>
+    <row r="13" spans="1:11" ht="316.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" s="2">
+        <v>1</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H13" s="2" t="s">
         <v>37</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="316.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" s="2">
-        <v>1</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>32</v>
       </c>
       <c r="I13" s="2">
         <v>1</v>
@@ -922,11 +964,151 @@
         <v>38</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>34</v>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="2">
+        <v>2</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I14" s="2">
+        <v>1</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="316.8" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="2">
+        <v>2</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="I15" s="2">
+        <v>1</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="345.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" s="2">
+        <v>2</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I16" s="2">
+        <v>5</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="345.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" s="2">
+        <v>2</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="I17" s="2">
+        <v>5</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K13" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:K13" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Core fix: Switched from generate_images → edit_image with SubjectReferenceImage(SUBJECT_TYPE_PRODUCT). The model now receives the   actual Meal tray red nobg.png cut-out and must place that exact product in the scene. No more text-description-only tray.
  Model: imagen-3.0-capability-001 — this is the model that supports the edit_image + product reference workflow.

  Product rules baked in: The subject_description explicitly says do not alter, recolor, or redesign — the same strict product rules
  the designers used.
</commit_message>
<xml_diff>
--- a/outputs/session_log.xlsx
+++ b/outputs/session_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ramakant\VSCode-projects\delicut-creative-workflow\outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85FAEFAC-4CE3-4561-8458-85B3DFAF4C81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7F1928C-1160-4F5B-A70F-3626D6E9B678}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="64">
   <si>
     <t>session_id</t>
   </si>
@@ -151,37 +151,286 @@
     <t>outputs\images\harry_0317-1622_locker-room-male_Imagen4Ultra.png</t>
   </si>
   <si>
+    <t xml:space="preserve">reject. Delicut product image and human features are not as per satisfaction. Ad copy doesn't seem to inherting or inspired from this image. </t>
+  </si>
+  <si>
     <t>Close-up of a single pair of athletic male hands on a dark gym floor. Left hand grips a clear protein shaker, right hand rests beside a 900ml square meal prep tray with warm beige base and clear lid with a bold red '/delicut/' label band. Both objects on the same surface, hands natural and relaxed. Single overhead studio light, deep clean shadows. No face visible. No other text. No other branding. Photorealistic, commercial photography, high contrast, sharp focus. 1080x1080.</t>
   </si>
   <si>
     <t>outputs\images\harry_0317-1622_hands-contrast_Imagen4Ultra.png</t>
   </si>
   <si>
+    <t>delicut meal box is empty without food which makes this very unlikely. Protein shaker is not placed properly</t>
+  </si>
+  <si>
     <t>Lean athletic female, mid-20s, running powerfully on a treadmill in a bright modern gym. Wearing a fitted sports bra and high-waist shorts with midriff visible. Hair tied back in a high ponytail, strong forward gaze, confident expression. Legs in mid-stride, slight motion blur suggesting speed. Bright overhead gym lighting, mirrors and equipment softly visible in background. Shot from a slight front-side angle at eye level. Natural athletic proportions, strong posture. No text. No branding. No logos. Photorealistic, energetic, shot on 50mm, bright and clean. 1080x1080.</t>
   </si>
   <si>
     <t>outputs\images\harry_0317-1622_treadmill-female_Imagen4Ultra.png</t>
   </si>
   <si>
+    <t>only concept that seems working</t>
+  </si>
+  <si>
+    <t>approved</t>
+  </si>
+  <si>
     <t>Top-down flat-lay on a deep spinach green surface, hex #043F12. Centre frame: a 900ml square meal prep tray with warm beige matte base, clear rigid plastic lid, bold red wraparound label band reading '/delicut/' in white. Arranged around it: a single white chalk-dusted weight plate, a neatly folded white gym towel, a stainless steel water bottle. Hard studio overhead lighting, crisp clean shadows, generous negative space. No additional text. No other branding. Commercial product photography, ultra-clean, high resolution. 1080x1080.</t>
   </si>
   <si>
     <t>outputs\images\harry_0317-1622_abstract-green_Imagen4Ultra.png</t>
   </si>
   <si>
-    <t xml:space="preserve">reject. Delicut product image and human features are not as per satisfaction. Ad copy doesn't seem to inherting or inspired from this image. </t>
-  </si>
-  <si>
-    <t>delicut meal box is empty without food which makes this very unlikely. Protein shaker is not placed properly</t>
-  </si>
-  <si>
-    <t>only concept that seems working</t>
-  </si>
-  <si>
     <t>this might work. But needs appropriate ad copy</t>
   </si>
   <si>
-    <t>approved</t>
+    <t>harry_0317-2328</t>
+  </si>
+  <si>
+    <t>SCENE:
+Modern commercial gym interior. Rows of treadmills, mirrors along one wall.
+Clean, well-lit space. Natural light from floor-to-ceiling windows on the left side.
+Background gym equipment and mirrors visible but softly out of focus.
+SUBJECT:
+Lean athletic female, mid-20s. Toned physique, natural proportions.
+Wearing a fitted sports bra and high-waist training shorts, midriff visible.
+Hair tied back in a high ponytail. Skin shows natural light sweat sheen.
+POSE:
+Running powerfully on a treadmill. Mid-stride, legs driving forward.
+Strong forward gaze — candid intensity, not posed. Slight motion blur on legs suggesting real speed.
+Natural weight distribution, forward lean of an actual runner.
+LIGHTING:
+Natural daylight from left-side floor-to-ceiling windows. Soft diffused light.
+Soft shadow falloff on the right side of the body. Clean balanced exposure.
+No overhead spot. No rim light.
+CAMERA:
+50mm equivalent. Eye-level angle, slightly front-side of the treadmill.
+Mid-thigh to head crop. Background softly blurred, gym context still readable.
+Use lifestyle/action camera settings.
+MOOD:
+Powerful, driven, in-the-zone. Energy of someone who makes no excuses.
+CAMERA SYSTEM:
+Canon R5 / Sony A7R IV. Natural lens perspective equivalent to 35mm–50mm full-frame.
+No wide-angle distortion. No telephoto compression.
+CAMERA SETTINGS (lifestyle / action):
+ISO 400. Shutter 1/1600 sec. Aperture f/4. Color temperature 5600K, neutral white balance.
+CAMERA SETTINGS (product flat-lay):
+ISO 200. Shutter 1/160 sec. Aperture f/2.8. Color temperature 5200K, neutral white balance.
+LIGHTING:
+Natural daylight only. No artificial flash, no studio strobes, no colored gels.
+Direction must be specified per scene. Quality defined as soft diffused or hard directional.
+Shadows are soft falloff or crisp depending on scene — described per variant above.
+Highlights are clean, not blown.
+COLOR TREATMENT:
+True-to-life color. Neutral whites — no yellow, orange, or blue cast.
+Balanced contrast — never cinematic or overgraded. No LUTs. No filters. No stylization.
+TEXTURE REALISM:
+Visible skin texture — natural pores, light sweat sheen where appropriate.
+Fabric shows natural behavior — wrinkles, stretch, folds at joints.
+Product surfaces show material texture — matte plastic, fabric weave, metal finish.
+DEPTH OF FIELD:
+Subject or hero product in sharp focus. Background softly blurred but contextually readable.
+COMPOSITION:
+Intentional but unstyled. Everything feels observed, not staged.
+Clear subject hierarchy. Use of negative space for premium, clean feel.
+No floating objects. Correct gravity, shadows, and light falloff.
+STRICT OUTPUT:
+No text overlays. No logos other than Delicut branding on product.
+No UI elements. No signage. Correct human anatomy and natural proportions.
+Ultra-high-definition editorial realism. Natural grain, not noise-free plastic look.</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0317-2328_treadmill-female_Imagen4Ultra.png</t>
+  </si>
+  <si>
+    <t>SCENE:
+Perfect overhead flat-lay on a deep spinach green surface, exact hex #043F12.
+Clean, minimal studio setup. Generous negative space. No background clutter.
+SUBJECT (HERO PRODUCT):
+Delicut 900ml meal prep tray — primary and dominant focus of the frame.
+Square form factor with soft rounded corners. Warm beige matte base.
+Clear rigid plastic lid. Bold red wraparound label band with '/delicut/' in white lettering.
+PRODUCT RULES:
+Do not alter, restyle, recolor, or redesign the tray. Maintain exact shape, material, and branding.
+Label must be clearly visible and readable.
+ARRANGEMENT:
+Tray centered in frame. At 10 o'clock: a single chalk-dusted white weight plate.
+At 4 o'clock: a neatly folded white gym towel. At 7 o'clock: a matte stainless steel water bottle.
+Each object naturally grounded with a realistic shadow beneath it.
+LIGHTING:
+Top-down overhead studio light. Hard directional, creating crisp clean shadows.
+No fill light. No colored gels. Color temperature 5200K.
+Use product flat-lay camera settings.
+CAMERA:
+50mm equivalent. Perfect 90-degree overhead angle, no perspective tilt.
+Objects fill approximately 70% of frame. Negative space is the green surface.
+MOOD:
+Clean, precise, performance-driven. Gym gear meets macro-perfect meal prep.
+CAMERA SYSTEM:
+Canon R5 / Sony A7R IV. Natural lens perspective equivalent to 35mm–50mm full-frame.
+No wide-angle distortion. No telephoto compression.
+CAMERA SETTINGS (lifestyle / action):
+ISO 400. Shutter 1/1600 sec. Aperture f/4. Color temperature 5600K, neutral white balance.
+CAMERA SETTINGS (product flat-lay):
+ISO 200. Shutter 1/160 sec. Aperture f/2.8. Color temperature 5200K, neutral white balance.
+LIGHTING:
+Natural daylight only. No artificial flash, no studio strobes, no colored gels.
+Direction must be specified per scene. Quality defined as soft diffused or hard directional.
+Shadows are soft falloff or crisp depending on scene — described per variant above.
+Highlights are clean, not blown.
+COLOR TREATMENT:
+True-to-life color. Neutral whites — no yellow, orange, or blue cast.
+Balanced contrast — never cinematic or overgraded. No LUTs. No filters. No stylization.
+TEXTURE REALISM:
+Visible skin texture — natural pores, light sweat sheen where appropriate.
+Fabric shows natural behavior — wrinkles, stretch, folds at joints.
+Product surfaces show material texture — matte plastic, fabric weave, metal finish.
+DEPTH OF FIELD:
+Subject or hero product in sharp focus. Background softly blurred but contextually readable.
+COMPOSITION:
+Intentional but unstyled. Everything feels observed, not staged.
+Clear subject hierarchy. Use of negative space for premium, clean feel.
+No floating objects. Correct gravity, shadows, and light falloff.
+STRICT OUTPUT:
+No text overlays. No logos other than Delicut branding on product.
+No UI elements. No signage. Correct human anatomy and natural proportions.
+Ultra-high-definition editorial realism. Natural grain, not noise-free plastic look.</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0317-2328_abstract-green_Imagen4Ultra.png</t>
+  </si>
+  <si>
+    <t>SCENE:
+Modern kitchen. Clean, minimal interior — white or light stone countertop visible.
+Refrigerator open in the background, interior light on. Time of day: morning.
+Natural light from a window to the left, soft and warm.
+SUBJECT:
+Athletic male, late 20s to early 30s. Lean but not bulky — fitness-conscious physique.
+Wearing a clean fitted white or grey t-shirt and training shorts.
+Natural, relaxed posture — not flexing, not posed.
+POSE:
+Reaching into the fridge or holding a Delicut 900ml meal prep tray at chest height.
+Looking at the tray with a natural satisfied expression — mid-moment, not smiling for camera.
+Weight shifted slightly to one leg. Arm extended naturally toward fridge.
+PRODUCT:
+Delicut 900ml meal prep tray. Warm beige matte base, clear rigid lid,
+bold red wraparound label reading '/delicut/' in white. Held naturally in one hand.
+Slight tilt from the grip — not perfectly horizontal. Fingers wrapped naturally around base.
+PRODUCT RULES:
+Do not alter tray design, color, or label. Label must be clearly readable.
+LIGHTING:
+Natural morning light from left window. Soft diffused quality. 5600K neutral white.
+Fridge interior light adds subtle warm fill from behind. No flash. No overhead spot.
+Soft shadow on right side of subject.
+CAMERA:
+35mm equivalent. Eye-level, slightly elevated angle.
+Three-quarter body shot — top of head to mid-thigh. Subject slightly left of center.
+Background kitchen and open fridge softly out of focus but readable.
+Use lifestyle/action camera settings.
+MOOD:
+Effortless healthy living. The fridge-smile moment — satisfaction without effort.
+CAMERA SYSTEM:
+Canon R5 / Sony A7R IV. Natural lens perspective equivalent to 35mm–50mm full-frame.
+No wide-angle distortion. No telephoto compression.
+CAMERA SETTINGS (lifestyle / action):
+ISO 400. Shutter 1/1600 sec. Aperture f/4. Color temperature 5600K, neutral white balance.
+CAMERA SETTINGS (product flat-lay):
+ISO 200. Shutter 1/160 sec. Aperture f/2.8. Color temperature 5200K, neutral white balance.
+LIGHTING:
+Natural daylight only. No artificial flash, no studio strobes, no colored gels.
+Direction must be specified per scene. Quality defined as soft diffused or hard directional.
+Shadows are soft falloff or crisp depending on scene — described per variant above.
+Highlights are clean, not blown.
+COLOR TREATMENT:
+True-to-life color. Neutral whites — no yellow, orange, or blue cast.
+Balanced contrast — never cinematic or overgraded. No LUTs. No filters. No stylization.
+TEXTURE REALISM:
+Visible skin texture — natural pores, light sweat sheen where appropriate.
+Fabric shows natural behavior — wrinkles, stretch, folds at joints.
+Product surfaces show material texture — matte plastic, fabric weave, metal finish.
+DEPTH OF FIELD:
+Subject or hero product in sharp focus. Background softly blurred but contextually readable.
+COMPOSITION:
+Intentional but unstyled. Everything feels observed, not staged.
+Clear subject hierarchy. Use of negative space for premium, clean feel.
+No floating objects. Correct gravity, shadows, and light falloff.
+STRICT OUTPUT:
+No text overlays. No logos other than Delicut branding on product.
+No UI elements. No signage. Correct human anatomy and natural proportions.
+Ultra-high-definition editorial realism. Natural grain, not noise-free plastic look.</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0317-2328_fridge-moment_Imagen4Ultra.png</t>
+  </si>
+  <si>
+    <t>SCENE:
+Gym locker room or quiet gym corner. Wooden bench in foreground.
+Lockers or a plain gym wall softly out of focus in background.
+Subdued, post-workout atmosphere — natural light from a high side window.
+SUBJECT:
+Athletic male, 28–32. Lean defined physique — not bulky, functionally fit.
+Wearing dark fitted compression shorts and a sleeveless training top.
+Natural post-workout state: slightly flushed, light sweat on arms and neck.
+POSE:
+Sitting on the bench. Forearms resting on knees, slight forward lean.
+Head slightly down, composed and focused — the stillness after a hard session.
+Not looking at camera. Hands relaxed, fingers loosely interlaced.
+PRODUCT (PRIMARY FOCUS):
+Delicut 900ml meal prep tray placed on the bench directly beside him — in sharp focus.
+Warm beige matte base, clear rigid lid, bold red '/delicut/' label clearly visible.
+Bag or gym kit partially visible beside tray, naturally suggesting he brought it for recovery.
+PRODUCT RULES:
+Tray is the sharpest element in the frame. Do not alter design, color, or label.
+Label must be clearly readable.
+LIGHTING:
+Natural side light from a high window. Single light source, slightly directional.
+Soft shadows across the locker room floor. Highlights on tray lid and subject's arms.
+No artificial fill. No rim light. 5600K neutral white.
+CAMERA:
+35mm equivalent. Low to mid angle — camera slightly below bench height.
+Focus on tray (sharp). Subject mid-ground, slightly blurred (depth of field).
+Mid-shot — bench surface to subject's shoulders. Tray occupies left third of frame.
+Use lifestyle/action camera settings.
+MOOD:
+Disciplined. Post-effort calm. The meal is the reward.
+CAMERA SYSTEM:
+Canon R5 / Sony A7R IV. Natural lens perspective equivalent to 35mm–50mm full-frame.
+No wide-angle distortion. No telephoto compression.
+CAMERA SETTINGS (lifestyle / action):
+ISO 400. Shutter 1/1600 sec. Aperture f/4. Color temperature 5600K, neutral white balance.
+CAMERA SETTINGS (product flat-lay):
+ISO 200. Shutter 1/160 sec. Aperture f/2.8. Color temperature 5200K, neutral white balance.
+LIGHTING:
+Natural daylight only. No artificial flash, no studio strobes, no colored gels.
+Direction must be specified per scene. Quality defined as soft diffused or hard directional.
+Shadows are soft falloff or crisp depending on scene — described per variant above.
+Highlights are clean, not blown.
+COLOR TREATMENT:
+True-to-life color. Neutral whites — no yellow, orange, or blue cast.
+Balanced contrast — never cinematic or overgraded. No LUTs. No filters. No stylization.
+TEXTURE REALISM:
+Visible skin texture — natural pores, light sweat sheen where appropriate.
+Fabric shows natural behavior — wrinkles, stretch, folds at joints.
+Product surfaces show material texture — matte plastic, fabric weave, metal finish.
+DEPTH OF FIELD:
+Subject or hero product in sharp focus. Background softly blurred but contextually readable.
+COMPOSITION:
+Intentional but unstyled. Everything feels observed, not staged.
+Clear subject hierarchy. Use of negative space for premium, clean feel.
+No floating objects. Correct gravity, shadows, and light falloff.
+STRICT OUTPUT:
+No text overlays. No logos other than Delicut branding on product.
+No UI elements. No signage. Correct human anatomy and natural proportions.
+Ultra-high-definition editorial realism. Natural grain, not noise-free plastic look.</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0317-2328_post-workout-bench_Imagen4Ultra.png</t>
+  </si>
+  <si>
+    <t>she's running the wrong way</t>
+  </si>
+  <si>
+    <t>meal tray is not as per specification</t>
   </si>
 </sst>
 </file>
@@ -538,7 +787,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="11" width="22" customWidth="1"/>
@@ -967,7 +1216,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>39</v>
       </c>
@@ -996,13 +1245,13 @@
         <v>1</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="316.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="316.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>39</v>
       </c>
@@ -1022,22 +1271,22 @@
         <v>15</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="I15" s="2">
         <v>1</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="K15" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="345.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="345.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>39</v>
       </c>
@@ -1057,22 +1306,22 @@
         <v>15</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I16" s="2">
         <v>5</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="345.6" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="345.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>39</v>
       </c>
@@ -1092,19 +1341,159 @@
         <v>15</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="I17" s="2">
         <v>5</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="2">
+        <v>3</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="I18" s="2">
+        <v>1</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" s="2">
+        <v>3</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="I19" s="2">
+        <v>1</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" s="2">
+        <v>3</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I20" s="2">
+        <v>1</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="K20" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="2">
+        <v>3</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="I21" s="2">
+        <v>1</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="K21" s="2">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
flux tried and rejected
</commit_message>
<xml_diff>
--- a/outputs/session_log.xlsx
+++ b/outputs/session_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ramakant\VSCode-projects\delicut-creative-workflow\outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55C24399-728B-4148-9A9F-DEF32D055783}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EA3ABFB-DA52-4B5C-A6EA-016FA2C71BE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="117">
   <si>
     <t>session_id</t>
   </si>
@@ -133,6 +133,9 @@
     <t>seems alright. Needs modification and alternatives</t>
   </si>
   <si>
+    <t>approved</t>
+  </si>
+  <si>
     <t>outputs\images\harry_0317-1502_abstract-green_Imagen4Ultra.png</t>
   </si>
   <si>
@@ -167,9 +170,6 @@
   </si>
   <si>
     <t>only concept that seems working</t>
-  </si>
-  <si>
-    <t>approved</t>
   </si>
   <si>
     <t>Top-down flat-lay on a deep spinach green surface, hex #043F12. Centre frame: a 900ml square meal prep tray with warm beige matte base, clear rigid plastic lid, bold red wraparound label band reading '/delicut/' in white. Arranged around it: a single white chalk-dusted weight plate, a neatly folded white gym towel, a stainless steel water bottle. Hard studio overhead lighting, crisp clean shadows, generous negative space. No additional text. No other branding. Commercial product photography, ultra-clean, high resolution. 1080x1080.</t>
@@ -439,6 +439,9 @@
     <t>ERROR: This method is only supported in the Vertex AI client.</t>
   </si>
   <si>
+    <t>not applicable</t>
+  </si>
+  <si>
     <t>harry_0318-0018</t>
   </si>
   <si>
@@ -451,28 +454,847 @@
     <t>outputs\images\harry_0318-0023_treadmill-female_Imagen3Capability.png</t>
   </si>
   <si>
+    <t>AI slop. There are 3 hands to this lady</t>
+  </si>
+  <si>
     <t>outputs\images\harry_0318-0023_abstract-green_Imagen3Capability.png</t>
   </si>
   <si>
+    <t>meal tray is not as per specification. Delicut is spelt as ellicut</t>
+  </si>
+  <si>
     <t>outputs\images\harry_0318-0023_fridge-moment_Imagen3Capability.png</t>
   </si>
   <si>
+    <t>AI slop. Fingers on the hand are incorrect. The delicut box is not as per reference image. It should be a green color box and not beige matte base. Correct this in the prompt</t>
+  </si>
+  <si>
     <t>outputs\images\harry_0318-0023_post-workout-bench_Imagen3Capability.png</t>
   </si>
   <si>
-    <t>not applicable</t>
-  </si>
-  <si>
-    <t>AI slop. There are 3 hands to this lady</t>
-  </si>
-  <si>
-    <t>meal tray is not as per specification. Delicut is spelt as ellicut</t>
-  </si>
-  <si>
-    <t>AI slop. Fingers on the hand are incorrect. The delicut box is not as per reference image. It should be a green color box and not beige matte base. Correct this in the prompt</t>
-  </si>
-  <si>
     <t>AI slop. The delicut logo and colors are completely wrong. Change box color to delicut green instead of beige matte</t>
+  </si>
+  <si>
+    <t>harry_0318-0034</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0318-0034_treadmill-female_Imagen3Capability.png</t>
+  </si>
+  <si>
+    <t>Delicut meal try is still not as per reference images. Meal cover is round. Slash is missing in the logo</t>
+  </si>
+  <si>
+    <t>SCENE:
+Perfect overhead flat-lay on a deep spinach green surface, exact hex #043F12.
+Clean, minimal studio setup. Generous negative space. No background clutter.
+SUBJECT (HERO PRODUCT):
+Delicut meal prep container — primary and dominant focus of the frame.
+Round shallow form factor. Deep spinach-green (#043F12) exterior sleeve.
+Bold white '/delicut' lettering wrapping the sides. Clear snap-on lid with silver rim edge.
+PRODUCT RULES:
+Do not alter, recolor, or redesign the container. Maintain exact green color and white branding.
+Label must be clearly visible and readable.
+ARRANGEMENT:
+Tray centered in frame. At 10 o'clock: a single chalk-dusted white weight plate.
+At 4 o'clock: a neatly folded white gym towel. At 7 o'clock: a matte stainless steel water bottle.
+Each object naturally grounded with a realistic shadow beneath it.
+LIGHTING:
+Top-down overhead studio light. Hard directional, creating crisp clean shadows.
+No fill light. No colored gels. Color temperature 5200K.
+Use product flat-lay camera settings.
+CAMERA:
+50mm equivalent. Perfect 90-degree overhead angle, no perspective tilt.
+Objects fill approximately 70% of frame. Negative space is the green surface.
+MOOD:
+Clean, precise, performance-driven. Gym gear meets macro-perfect meal prep.
+CAMERA SYSTEM:
+Canon R5 / Sony A7R IV. Natural lens perspective equivalent to 35mm–50mm full-frame.
+No wide-angle distortion. No telephoto compression.
+CAMERA SETTINGS (lifestyle / action):
+ISO 400. Shutter 1/1600 sec. Aperture f/4. Color temperature 5600K, neutral white balance.
+CAMERA SETTINGS (product flat-lay):
+ISO 200. Shutter 1/160 sec. Aperture f/2.8. Color temperature 5200K, neutral white balance.
+LIGHTING:
+Natural daylight only. No artificial flash, no studio strobes, no colored gels.
+Direction must be specified per scene. Quality defined as soft diffused or hard directional.
+Shadows are soft falloff or crisp depending on scene — described per variant above.
+Highlights are clean, not blown.
+COLOR TREATMENT:
+True-to-life color. Neutral whites — no yellow, orange, or blue cast.
+Balanced contrast — never cinematic or overgraded. No LUTs. No filters. No stylization.
+TEXTURE REALISM:
+Visible skin texture — natural pores, light sweat sheen where appropriate.
+Fabric shows natural behavior — wrinkles, stretch, folds at joints.
+Product surfaces show material texture — matte plastic, fabric weave, metal finish.
+DEPTH OF FIELD:
+Subject or hero product in sharp focus. Background softly blurred but contextually readable.
+COMPOSITION:
+Intentional but unstyled. Everything feels observed, not staged.
+Clear subject hierarchy. Use of negative space for premium, clean feel.
+No floating objects. Correct gravity, shadows, and light falloff.
+STRICT OUTPUT:
+No text overlays. No logos other than Delicut branding on product.
+No UI elements. No signage. Correct human anatomy and natural proportions.
+Ultra-high-definition editorial realism. Natural grain, not noise-free plastic look.</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0318-0034_abstract-green_Imagen3Capability.png</t>
+  </si>
+  <si>
+    <t>meal box is incorrect. AI slop as boxes are hanging in mid-air</t>
+  </si>
+  <si>
+    <t>SCENE:
+Modern kitchen. Clean, minimal interior — white or light stone countertop visible.
+Refrigerator open in the background, interior light on. Time of day: morning.
+Natural light from a window to the left, soft and warm.
+SUBJECT:
+Athletic male, late 20s to early 30s. Lean but not bulky — fitness-conscious physique.
+Wearing a clean fitted white or grey t-shirt and training shorts.
+Natural, relaxed posture — not flexing, not posed.
+POSE:
+Reaching into the fridge or holding a Delicut 900ml meal prep tray at chest height.
+Looking at the tray with a natural satisfied expression — mid-moment, not smiling for camera.
+Weight shifted slightly to one leg. Arm extended naturally toward fridge.
+PRODUCT:
+Delicut meal prep container. Round shallow form factor, deep spinach-green (#043F12) exterior
+printed with '/delicut' in bold white lettering. Clear snap-on lid with silver rim.
+Held naturally in one hand. Slight tilt from grip. Fingers wrapped naturally around base.
+PRODUCT RULES:
+Do not alter tray design, color, or label. Label must be clearly readable.
+LIGHTING:
+Natural morning light from left window. Soft diffused quality. 5600K neutral white.
+Fridge interior light adds subtle warm fill from behind. No flash. No overhead spot.
+Soft shadow on right side of subject.
+CAMERA:
+35mm equivalent. Eye-level, slightly elevated angle.
+Three-quarter body shot — top of head to mid-thigh. Subject slightly left of center.
+Background kitchen and open fridge softly out of focus but readable.
+Use lifestyle/action camera settings.
+MOOD:
+Effortless healthy living. The fridge-smile moment — satisfaction without effort.
+CAMERA SYSTEM:
+Canon R5 / Sony A7R IV. Natural lens perspective equivalent to 35mm–50mm full-frame.
+No wide-angle distortion. No telephoto compression.
+CAMERA SETTINGS (lifestyle / action):
+ISO 400. Shutter 1/1600 sec. Aperture f/4. Color temperature 5600K, neutral white balance.
+CAMERA SETTINGS (product flat-lay):
+ISO 200. Shutter 1/160 sec. Aperture f/2.8. Color temperature 5200K, neutral white balance.
+LIGHTING:
+Natural daylight only. No artificial flash, no studio strobes, no colored gels.
+Direction must be specified per scene. Quality defined as soft diffused or hard directional.
+Shadows are soft falloff or crisp depending on scene — described per variant above.
+Highlights are clean, not blown.
+COLOR TREATMENT:
+True-to-life color. Neutral whites — no yellow, orange, or blue cast.
+Balanced contrast — never cinematic or overgraded. No LUTs. No filters. No stylization.
+TEXTURE REALISM:
+Visible skin texture — natural pores, light sweat sheen where appropriate.
+Fabric shows natural behavior — wrinkles, stretch, folds at joints.
+Product surfaces show material texture — matte plastic, fabric weave, metal finish.
+DEPTH OF FIELD:
+Subject or hero product in sharp focus. Background softly blurred but contextually readable.
+COMPOSITION:
+Intentional but unstyled. Everything feels observed, not staged.
+Clear subject hierarchy. Use of negative space for premium, clean feel.
+No floating objects. Correct gravity, shadows, and light falloff.
+STRICT OUTPUT:
+No text overlays. No logos other than Delicut branding on product.
+No UI elements. No signage. Correct human anatomy and natural proportions.
+Ultra-high-definition editorial realism. Natural grain, not noise-free plastic look.</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0318-0034_fridge-moment_Imagen3Capability.png</t>
+  </si>
+  <si>
+    <t>human image is portrayed correctly but delicut box is completely wrong. The spinach color is correct but delicut logo is missing slash at the end. Dimensions and shape of box are wrong</t>
+  </si>
+  <si>
+    <t>SCENE:
+Gym locker room or quiet gym corner. Wooden bench in foreground.
+Lockers or a plain gym wall softly out of focus in background.
+Subdued, post-workout atmosphere — natural light from a high side window.
+SUBJECT:
+Athletic male, 28–32. Lean defined physique — not bulky, functionally fit.
+Wearing dark fitted compression shorts and a sleeveless training top.
+Natural post-workout state: slightly flushed, light sweat on arms and neck.
+POSE:
+Sitting on the bench. Forearms resting on knees, slight forward lean.
+Head slightly down, composed and focused — the stillness after a hard session.
+Not looking at camera. Hands relaxed, fingers loosely interlaced.
+PRODUCT (PRIMARY FOCUS):
+Delicut meal prep container placed on the bench directly beside him — in sharp focus.
+Round, deep spinach-green (#043F12) exterior with '/delicut' in bold white lettering, clear snap-on lid.
+Gym kit partially visible beside it, naturally suggesting he brought it for recovery.
+PRODUCT RULES:
+Container is the sharpest element in the frame. Do not alter design, color, or branding.
+Green exterior and white '/delicut' text must be clearly readable.
+LIGHTING:
+Natural side light from a high window. Single light source, slightly directional.
+Soft shadows across the locker room floor. Highlights on tray lid and subject's arms.
+No artificial fill. No rim light. 5600K neutral white.
+CAMERA:
+35mm equivalent. Low to mid angle — camera slightly below bench height.
+Focus on tray (sharp). Subject mid-ground, slightly blurred (depth of field).
+Mid-shot — bench surface to subject's shoulders. Tray occupies left third of frame.
+Use lifestyle/action camera settings.
+MOOD:
+Disciplined. Post-effort calm. The meal is the reward.
+CAMERA SYSTEM:
+Canon R5 / Sony A7R IV. Natural lens perspective equivalent to 35mm–50mm full-frame.
+No wide-angle distortion. No telephoto compression.
+CAMERA SETTINGS (lifestyle / action):
+ISO 400. Shutter 1/1600 sec. Aperture f/4. Color temperature 5600K, neutral white balance.
+CAMERA SETTINGS (product flat-lay):
+ISO 200. Shutter 1/160 sec. Aperture f/2.8. Color temperature 5200K, neutral white balance.
+LIGHTING:
+Natural daylight only. No artificial flash, no studio strobes, no colored gels.
+Direction must be specified per scene. Quality defined as soft diffused or hard directional.
+Shadows are soft falloff or crisp depending on scene — described per variant above.
+Highlights are clean, not blown.
+COLOR TREATMENT:
+True-to-life color. Neutral whites — no yellow, orange, or blue cast.
+Balanced contrast — never cinematic or overgraded. No LUTs. No filters. No stylization.
+TEXTURE REALISM:
+Visible skin texture — natural pores, light sweat sheen where appropriate.
+Fabric shows natural behavior — wrinkles, stretch, folds at joints.
+Product surfaces show material texture — matte plastic, fabric weave, metal finish.
+DEPTH OF FIELD:
+Subject or hero product in sharp focus. Background softly blurred but contextually readable.
+COMPOSITION:
+Intentional but unstyled. Everything feels observed, not staged.
+Clear subject hierarchy. Use of negative space for premium, clean feel.
+No floating objects. Correct gravity, shadows, and light falloff.
+STRICT OUTPUT:
+No text overlays. No logos other than Delicut branding on product.
+No UI elements. No signage. Correct human anatomy and natural proportions.
+Ultra-high-definition editorial realism. Natural grain, not noise-free plastic look.</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0318-0034_post-workout-bench_Imagen3Capability.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">woman anatomy is correct but she's running in the wrong way. Humans run along the treadmill. She has been placed runnning sideways on the treadmill </t>
+  </si>
+  <si>
+    <t>harry_0318-0103</t>
+  </si>
+  <si>
+    <t>SCENE:
+Modern commercial gym interior. Rows of treadmills, mirrors along one wall.
+Clean, well-lit space. Natural light from floor-to-ceiling windows on the left side.
+Background gym equipment and mirrors visible but softly out of focus.
+SUBJECT:
+Lean athletic female, mid-20s. Toned physique, natural proportions.
+Wearing a fitted sports bra and high-waist training shorts, midriff visible.
+Hair tied back in a high ponytail. Skin shows natural light sweat sheen.
+POSE:
+Running powerfully on a treadmill with body facing front. Mid-stride, legs driving forward.
+Strong forward gaze â€” candid intensity, not posed. Slight motion blur on legs suggesting real speed.
+Natural weight distribution, forward lean of an actual runner.
+PRODUCT:
+Delicut meal prep container. Round shallow form factor.
+Deep spinach-green (#043F12) exterior with bold white sans-serif text repeating around the full
+circumference: /delicut /delicut /delicut — forward slash before and after each instance.
+Clear snap-on plastic lid with a silver rim edge.
+LID LABEL:
+A white square adhesive label (approx 60x60mm) sits centered on the clear lid, showing:
+- Top-left: /delicut/ logo in bold sans-serif. Top-right: delicut.ae URL
+- Dish name in large bold text (e.g. Grilled Chicken and Roasted Vegetables)
+- Meal category (e.g. High Protein Main)
+- Macro grid: kcal 480 | pro 42 | carbs 28 | fat 14
+- Customer first name, best before date, barcode at bottom
+Label text is crisp black on white, clean typographic layout.
+FOOD INSIDE:
+Visible through the clear lid — grilled chicken breast sliced on the diagonal,
+roasted broccoli and capsicum, a portion of fluffy quinoa. Vibrant, appetising colours
+through the clear plastic. Moisture on the vegetables catching light.
+PRODUCT RULES:
+- Container exterior must be deep spinach-green (#043F12) — not beige, not red, not brown
+- /delicut/ branding in white, forward slashes on both sides, clearly readable
+- Lid label must be white with black text, macro grid visible
+- Do not alter, recolor, or redesign any element
+LIGHTING:
+Natural daylight from left-side floor-to-ceiling windows. Soft diffused light.
+Soft shadow falloff on the right side of the body. Clean balanced exposure.
+No overhead spot. No rim light.
+CAMERA:
+50mm equivalent. Eye-level angle, slightly front-side of the treadmill.
+Mid-thigh to head crop. Background softly blurred, gym context still readable.
+Use lifestyle/action camera settings.
+MOOD:
+Powerful, driven, in-the-zone. Energy of someone who makes no excuses.
+CAMERA SYSTEM:
+Canon R5 / Sony A7R IV. Natural lens perspective equivalent to 35mmâ€“50mm full-frame.
+No wide-angle distortion. No telephoto compression.
+CAMERA SETTINGS (lifestyle / action):
+ISO 400. Shutter 1/1600 sec. Aperture f/4. Color temperature 5600K, neutral white balance.
+CAMERA SETTINGS (product flat-lay):
+ISO 200. Shutter 1/160 sec. Aperture f/2.8. Color temperature 5200K, neutral white balance.
+LIGHTING:
+Natural daylight only. No artificial flash, no studio strobes, no colored gels.
+Direction must be specified per scene. Quality defined as soft diffused or hard directional.
+Shadows are soft falloff or crisp depending on scene â€” described per variant above.
+Highlights are clean, not blown.
+COLOR TREATMENT:
+True-to-life color. Neutral whites â€” no yellow, orange, or blue cast.
+Balanced contrast â€” never cinematic or overgraded. No LUTs. No filters. No stylization.
+TEXTURE REALISM:
+Visible skin texture â€” natural pores, light sweat sheen where appropriate.
+Fabric shows natural behavior â€” wrinkles, stretch, folds at joints.
+Product surfaces show material texture â€” matte plastic, fabric weave, metal finish.
+DEPTH OF FIELD:
+Subject or hero product in sharp focus. Background softly blurred but contextually readable.
+COMPOSITION:
+Intentional but unstyled. Everything feels observed, not staged.
+Clear subject hierarchy. Use of negative space for premium, clean feel.
+No floating objects. Correct gravity, shadows, and light falloff.
+STRICT OUTPUT:
+No text overlays. No logos other than Delicut branding on product.
+No UI elements. No signage. Correct human anatomy and natural proportions.
+Ultra-high-definition editorial realism. Natural grain, not noise-free plastic look.</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0318-0103_treadmill-female_Imagen3Capability.png</t>
+  </si>
+  <si>
+    <t>product was never supposed to be shown in the runner. This needs to be remove</t>
+  </si>
+  <si>
+    <t>SCENE:
+Perfect overhead flat-lay on a deep spinach green surface, exact hex #043F12.
+Clean, minimal studio setup. Generous negative space. No background clutter.
+ARRANGEMENT:
+Tray centered in frame. At 10 o'clock: a single chalk-dusted white weight plate.
+At 4 o'clock: a neatly folded white gym towel. At 7 o'clock: a matte stainless steel water bottle.
+Each object naturally grounded with a realistic shadow beneath it.
+PRODUCT:
+Delicut meal prep container. Round shallow form factor.
+Deep spinach-green (#043F12) exterior with bold white sans-serif text repeating around the full
+circumference: /delicut /delicut /delicut — forward slash before and after each instance.
+Clear snap-on plastic lid with a silver rim edge.
+LID LABEL:
+A white square adhesive label (approx 60x60mm) sits centered on the clear lid, showing:
+- Top-left: /delicut/ logo in bold sans-serif. Top-right: delicut.ae URL
+- Dish name in large bold text (e.g. Grilled Chicken and Roasted Vegetables)
+- Meal category (e.g. High Protein Main)
+- Macro grid: kcal 480 | pro 42 | carbs 28 | fat 14
+- Customer first name, best before date, barcode at bottom
+Label text is crisp black on white, clean typographic layout.
+FOOD INSIDE:
+Visible through the clear lid — grilled chicken breast sliced on the diagonal,
+roasted broccoli and capsicum, a portion of fluffy quinoa. Vibrant, appetising colours
+through the clear plastic. Moisture on the vegetables catching light.
+PRODUCT RULES:
+- Container exterior must be deep spinach-green (#043F12) — not beige, not red, not brown
+- /delicut/ branding in white, forward slashes on both sides, clearly readable
+- Lid label must be white with black text, macro grid visible
+- Do not alter, recolor, or redesign any element
+LIGHTING:
+Top-down overhead studio light. Hard directional, creating crisp clean shadows.
+No fill light. No colored gels. Color temperature 5200K.
+Use product flat-lay camera settings.
+CAMERA:
+50mm equivalent. Perfect 90-degree overhead angle, no perspective tilt.
+Objects fill approximately 70% of frame. Negative space is the green surface.
+MOOD:
+Clean, precise, performance-driven. Gym gear meets macro-perfect meal prep.
+CAMERA SYSTEM:
+Canon R5 / Sony A7R IV. Natural lens perspective equivalent to 35mmâ€“50mm full-frame.
+No wide-angle distortion. No telephoto compression.
+CAMERA SETTINGS (lifestyle / action):
+ISO 400. Shutter 1/1600 sec. Aperture f/4. Color temperature 5600K, neutral white balance.
+CAMERA SETTINGS (product flat-lay):
+ISO 200. Shutter 1/160 sec. Aperture f/2.8. Color temperature 5200K, neutral white balance.
+LIGHTING:
+Natural daylight only. No artificial flash, no studio strobes, no colored gels.
+Direction must be specified per scene. Quality defined as soft diffused or hard directional.
+Shadows are soft falloff or crisp depending on scene â€” described per variant above.
+Highlights are clean, not blown.
+COLOR TREATMENT:
+True-to-life color. Neutral whites â€” no yellow, orange, or blue cast.
+Balanced contrast â€” never cinematic or overgraded. No LUTs. No filters. No stylization.
+TEXTURE REALISM:
+Visible skin texture â€” natural pores, light sweat sheen where appropriate.
+Fabric shows natural behavior â€” wrinkles, stretch, folds at joints.
+Product surfaces show material texture â€” matte plastic, fabric weave, metal finish.
+DEPTH OF FIELD:
+Subject or hero product in sharp focus. Background softly blurred but contextually readable.
+COMPOSITION:
+Intentional but unstyled. Everything feels observed, not staged.
+Clear subject hierarchy. Use of negative space for premium, clean feel.
+No floating objects. Correct gravity, shadows, and light falloff.
+STRICT OUTPUT:
+No text overlays. No logos other than Delicut branding on product.
+No UI elements. No signage. Correct human anatomy and natural proportions.
+Ultra-high-definition editorial realism. Natural grain, not noise-free plastic look.</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0318-0103_abstract-green_Imagen3Capability.png</t>
+  </si>
+  <si>
+    <t>label dimensions are incoorect. Box dimensions are incorrect. Remove black borders. Label imagery needs to be followed more strictly. Rendering of the label is inconsistent and incomplete. Text on label is unreadable. Food appears outside the box. Tray is a bit too transparent. needs to be slightly opaque</t>
+  </si>
+  <si>
+    <t>SCENE:
+Modern kitchen. Clean, minimal interior â€” white or light stone countertop visible.
+Refrigerator open in the background, interior light on. Time of day: morning.
+Natural light from a window to the left, soft and warm.
+SUBJECT:
+Athletic male, late 20s to early 30s. Lean but not bulky â€” fitness-conscious physique.
+Wearing a clean fitted white or grey t-shirt and training shorts.
+Natural, relaxed posture â€” not flexing, not posed.
+POSE:
+Reaching into the fridge or holding a Delicut 900ml meal prep tray at chest height.
+Looking at the tray with a natural satisfied expression â€” mid-moment, not smiling for camera.
+Weight shifted slightly to one leg. Arm extended naturally toward fridge.
+PRODUCT:
+Delicut meal prep container. Round shallow form factor.
+Deep spinach-green (#043F12) exterior with bold white sans-serif text repeating around the full
+circumference: /delicut /delicut /delicut — forward slash before and after each instance.
+Clear snap-on plastic lid with a silver rim edge.
+LID LABEL:
+A white square adhesive label (approx 60x60mm) sits centered on the clear lid, showing:
+- Top-left: /delicut/ logo in bold sans-serif. Top-right: delicut.ae URL
+- Dish name in large bold text (e.g. Grilled Chicken and Roasted Vegetables)
+- Meal category (e.g. High Protein Main)
+- Macro grid: kcal 480 | pro 42 | carbs 28 | fat 14
+- Customer first name, best before date, barcode at bottom
+Label text is crisp black on white, clean typographic layout.
+FOOD INSIDE:
+Visible through the clear lid — grilled chicken breast sliced on the diagonal,
+roasted broccoli and capsicum, a portion of fluffy quinoa. Vibrant, appetising colours
+through the clear plastic. Moisture on the vegetables catching light.
+PRODUCT RULES:
+- Container exterior must be deep spinach-green (#043F12) — not beige, not red, not brown
+- /delicut/ branding in white, forward slashes on both sides, clearly readable
+- Lid label must be white with black text, macro grid visible
+- Do not alter, recolor, or redesign any element
+LIGHTING:
+Natural morning light from left window. Soft diffused quality. 5600K neutral white.
+Fridge interior light adds subtle warm fill from behind. No flash. No overhead spot.
+Soft shadow on right side of subject.
+CAMERA:
+35mm equivalent. Eye-level, slightly elevated angle.
+Three-quarter body shot â€” top of head to mid-thigh. Subject slightly left of center.
+Background kitchen and open fridge softly out of focus but readable.
+Use lifestyle/action camera settings.
+MOOD:
+Effortless healthy living. The fridge-smile moment â€” satisfaction without effort.
+CAMERA SYSTEM:
+Canon R5 / Sony A7R IV. Natural lens perspective equivalent to 35mmâ€“50mm full-frame.
+No wide-angle distortion. No telephoto compression.
+CAMERA SETTINGS (lifestyle / action):
+ISO 400. Shutter 1/1600 sec. Aperture f/4. Color temperature 5600K, neutral white balance.
+CAMERA SETTINGS (product flat-lay):
+ISO 200. Shutter 1/160 sec. Aperture f/2.8. Color temperature 5200K, neutral white balance.
+LIGHTING:
+Natural daylight only. No artificial flash, no studio strobes, no colored gels.
+Direction must be specified per scene. Quality defined as soft diffused or hard directional.
+Shadows are soft falloff or crisp depending on scene â€” described per variant above.
+Highlights are clean, not blown.
+COLOR TREATMENT:
+True-to-life color. Neutral whites â€” no yellow, orange, or blue cast.
+Balanced contrast â€” never cinematic or overgraded. No LUTs. No filters. No stylization.
+TEXTURE REALISM:
+Visible skin texture â€” natural pores, light sweat sheen where appropriate.
+Fabric shows natural behavior â€” wrinkles, stretch, folds at joints.
+Product surfaces show material texture â€” matte plastic, fabric weave, metal finish.
+DEPTH OF FIELD:
+Subject or hero product in sharp focus. Background softly blurred but contextually readable.
+COMPOSITION:
+Intentional but unstyled. Everything feels observed, not staged.
+Clear subject hierarchy. Use of negative space for premium, clean feel.
+No floating objects. Correct gravity, shadows, and light falloff.
+STRICT OUTPUT:
+No text overlays. No logos other than Delicut branding on product.
+No UI elements. No signage. Correct human anatomy and natural proportions.
+Ultra-high-definition editorial realism. Natural grain, not noise-free plastic look.</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0318-0103_fridge-moment_Imagen3Capability.png</t>
+  </si>
+  <si>
+    <t>delicut box is rendered correctly but the label is incorrect. It should come on the top of the lid and not sideways. if the box is being viewd from the side, then the label should not be seen. Pose, scene and subject are all correct. Image is over-saturated and too many shadows</t>
+  </si>
+  <si>
+    <t>SCENE:
+Gym locker room or quiet gym corner. Wooden bench in foreground.
+Lockers or a plain gym wall softly out of focus in background.
+Subdued, post-workout atmosphere â€” natural light from a high side window.
+SUBJECT:
+Athletic male, 28â€“32. Lean defined physique â€” not bulky, functionally fit.
+Wearing dark fitted compression shorts and a sleeveless training top.
+Natural post-workout state: slightly flushed, light sweat on arms and neck.
+POSE:
+Sitting on the bench. Forearms resting on knees, slight forward lean.
+Head slightly down, composed and focused â€” the stillness after a hard session.
+Not looking at camera. Hands relaxed, fingers loosely interlaced.
+PRODUCT:
+Delicut meal prep container. Round shallow form factor.
+Deep spinach-green (#043F12) exterior with bold white sans-serif text repeating around the full
+circumference: /delicut /delicut /delicut — forward slash before and after each instance.
+Clear snap-on plastic lid with a silver rim edge.
+LID LABEL:
+A white square adhesive label (approx 60x60mm) sits centered on the clear lid, showing:
+- Top-left: /delicut/ logo in bold sans-serif. Top-right: delicut.ae URL
+- Dish name in large bold text (e.g. Grilled Chicken and Roasted Vegetables)
+- Meal category (e.g. High Protein Main)
+- Macro grid: kcal 480 | pro 42 | carbs 28 | fat 14
+- Customer first name, best before date, barcode at bottom
+Label text is crisp black on white, clean typographic layout.
+FOOD INSIDE:
+Visible through the clear lid — grilled chicken breast sliced on the diagonal,
+roasted broccoli and capsicum, a portion of fluffy quinoa. Vibrant, appetising colours
+through the clear plastic. Moisture on the vegetables catching light.
+PRODUCT RULES:
+- Container exterior must be deep spinach-green (#043F12) — not beige, not red, not brown
+- /delicut/ branding in white, forward slashes on both sides, clearly readable
+- Lid label must be white with black text, macro grid visible
+- Do not alter, recolor, or redesign any element
+LIGHTING:
+Natural side light from a high window. Single light source, slightly directional.
+Soft shadows across the locker room floor. Highlights on tray lid and subject's arms.
+No artificial fill. No rim light. 5600K neutral white.
+CAMERA:
+35mm equivalent. Low to mid angle â€” camera slightly below bench height.
+Focus on tray (sharp). Subject mid-ground, slightly blurred (depth of field).
+Mid-shot â€” bench surface to subject's shoulders. Tray occupies left third of frame.
+Use lifestyle/action camera settings.
+MOOD:
+Disciplined. Post-effort calm. The meal is the reward.
+CAMERA SYSTEM:
+Canon R5 / Sony A7R IV. Natural lens perspective equivalent to 35mmâ€“50mm full-frame.
+No wide-angle distortion. No telephoto compression.
+CAMERA SETTINGS (lifestyle / action):
+ISO 400. Shutter 1/1600 sec. Aperture f/4. Color temperature 5600K, neutral white balance.
+CAMERA SETTINGS (product flat-lay):
+ISO 200. Shutter 1/160 sec. Aperture f/2.8. Color temperature 5200K, neutral white balance.
+LIGHTING:
+Natural daylight only. No artificial flash, no studio strobes, no colored gels.
+Direction must be specified per scene. Quality defined as soft diffused or hard directional.
+Shadows are soft falloff or crisp depending on scene â€” described per variant above.
+Highlights are clean, not blown.
+COLOR TREATMENT:
+True-to-life color. Neutral whites â€” no yellow, orange, or blue cast.
+Balanced contrast â€” never cinematic or overgraded. No LUTs. No filters. No stylization.
+TEXTURE REALISM:
+Visible skin texture â€” natural pores, light sweat sheen where appropriate.
+Fabric shows natural behavior â€” wrinkles, stretch, folds at joints.
+Product surfaces show material texture â€” matte plastic, fabric weave, metal finish.
+DEPTH OF FIELD:
+Subject or hero product in sharp focus. Background softly blurred but contextually readable.
+COMPOSITION:
+Intentional but unstyled. Everything feels observed, not staged.
+Clear subject hierarchy. Use of negative space for premium, clean feel.
+No floating objects. Correct gravity, shadows, and light falloff.
+STRICT OUTPUT:
+No text overlays. No logos other than Delicut branding on product.
+No UI elements. No signage. Correct human anatomy and natural proportions.
+Ultra-high-definition editorial realism. Natural grain, not noise-free plastic look.</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0318-0103_post-workout-bench_Imagen3Capability.png</t>
+  </si>
+  <si>
+    <t>meal box dimensions in relation to human are incorrect. The delicut on the box sides should be in a single line. Font is incorrect. If customer name is not clear, generate a customer name in the prompt for clear instruction</t>
+  </si>
+  <si>
+    <t>pending</t>
+  </si>
+  <si>
+    <t>harry_0318-0125</t>
+  </si>
+  <si>
+    <t>Flux1Pro</t>
+  </si>
+  <si>
+    <t>SCENE:
+Modern commercial gym interior. Rows of treadmills, mirrors along one wall.
+Clean, well-lit space. Natural light from floor-to-ceiling windows on the left side.
+Background gym equipment and mirrors visible but softly out of focus.
+SUBJECT:
+Lean athletic female, mid-20s. Toned physique, natural proportions.
+Wearing a fitted sports bra and high-waist training shorts, midriff visible.
+Hair tied back in a high ponytail. Skin shows natural light sweat sheen.
+POSE:
+Running powerfully on a treadmill with body facing front. Mid-stride, legs driving forward.
+Strong forward gaze — candid intensity, not posed. Slight motion blur on legs suggesting real speed.
+Natural weight distribution, forward lean of an actual runner. Running direction is ALONG the treadmill, not sideways.
+NO PRODUCT in this image. No meal containers, no food packaging, no Delicut boxes.
+Pure lifestyle runner shot — subject and gym environment only.
+LIGHTING:
+Natural daylight from left-side floor-to-ceiling windows. Soft diffused light.
+Soft shadow falloff on the right side of the body. Clean balanced exposure.
+No overhead spot. No rim light.
+CAMERA:
+50mm equivalent. Eye-level angle, slightly front-side of the treadmill.
+Mid-thigh to head crop. Background softly blurred, gym context still readable.
+Use lifestyle/action camera settings.
+MOOD:
+Powerful, driven, in-the-zone. Energy of someone who makes no excuses.
+CAMERA SYSTEM:
+Canon R5 / Sony A7R IV. Natural lens perspective equivalent to 35mm-50mm full-frame.
+No wide-angle distortion. No telephoto compression.
+CAMERA SETTINGS (lifestyle / action):
+ISO 400. Shutter 1/1600 sec. Aperture f/4. Color temperature 5600K, neutral white balance.
+LIGHTING:
+Natural daylight only. No artificial flash, no studio strobes, no colored gels.
+Direction must be specified per scene. Quality defined as soft diffused or hard directional.
+Shadows are soft falloff. Highlights are clean, not blown.
+COLOR TREATMENT:
+True-to-life color. Neutral whites — no yellow, orange, or blue cast.
+Balanced contrast — never cinematic or overgraded. No LUTs. No filters. No stylization.
+TEXTURE REALISM:
+Visible skin texture — natural pores, light sweat sheen where appropriate.
+Fabric shows natural behavior — wrinkles, stretch, folds at joints.
+DEPTH OF FIELD:
+Subject in sharp focus. Background softly blurred but contextually readable.
+COMPOSITION:
+Intentional but unstyled. Everything feels observed, not staged.
+Clear subject hierarchy. Use of negative space for premium, clean feel.
+No floating objects. Correct gravity, shadows, and light falloff.
+STRICT OUTPUT:
+No text overlays. No logos. No UI elements. No signage. No food packaging.
+Correct human anatomy and natural proportions.
+Ultra-high-definition editorial realism. Natural grain, not noise-free plastic look.</t>
+  </si>
+  <si>
+    <t>ERROR: Prediction failed: Error generating image: NSFW content detected.</t>
+  </si>
+  <si>
+    <t>SCENE:
+Perfect overhead flat-lay on a deep spinach green surface, exact hex #043F12.
+Clean, minimal studio setup. Generous negative space. No background clutter. No black borders.
+ARRANGEMENT:
+Tray centered in frame. At 10 o'clock: a single chalk-dusted white weight plate.
+At 4 o'clock: a neatly folded white gym towel. At 7 o'clock: a matte stainless steel water bottle.
+Each object naturally grounded with a realistic shadow beneath it.
+PRODUCT:
+Delicut meal prep container. Round shallow form factor, approximately 18cm diameter and 6cm tall.
+Deep spinach-green (#043F12) exterior sleeve printed with /delicut/ in bold white sans-serif lettering.
+SLIGHTLY OPAQUE frosted lid — not fully transparent, not opaque. A frosted/translucent finish.
+Silver rim edge around the lid. No black borders on any part of the container.
+LID LABEL:
+A white square adhesive label exactly 60x60mm sits perfectly centered on the TOP of the frosted lid.
+The label is FLAT on the top surface — never wrapped around the sides.
+Label contents:
+- Top-left corner: /delicut/ logo in bold sans-serif (8pt). Top-right corner: delicut.ae URL (7pt)
+- Center: Dish name in large bold text — "Grilled Chicken &amp; Roasted Vegetables" (12pt)
+- Below dish name: Meal category — "High Protein Main" (9pt)
+- Macro row: kcal 480 | pro 42g | carbs 28g | fat 14g (8pt, evenly spaced)
+- Bottom row: Customer name "Ahmed Al Mansoori" | best before date | barcode
+All text is crisp black on white. Clean typographic layout. All text must be legible.
+FOOD INSIDE:
+Food is FULLY CONTAINED inside the tray — nothing spilling out or extending beyond the rim.
+Visible through the slightly frosted lid: grilled chicken breast sliced on the diagonal,
+roasted broccoli and capsicum, a portion of fluffy quinoa. Vibrant, appetising colours.
+Moisture on the vegetables catching light. Food fills the container but does not overflow.
+PRODUCT RULES:
+- Container exterior must be deep spinach-green (#043F12) — not beige, not red, not brown
+- /delicut/ branding in white, forward slashes on both sides, clearly readable
+- Lid must be slightly opaque/frosted — not clear, not solid
+- Lid label flat on top only — never sideways, never on the rim
+- No black borders anywhere
+- Container diameter approximately 18cm — realistic food container scale
+- Do not alter, recolor, or redesign any element of the container
+LIGHTING:
+Top-down overhead studio light. Hard directional, creating crisp clean shadows.
+No fill light. No colored gels. Color temperature 5200K.
+Use product flat-lay camera settings.
+CAMERA:
+50mm equivalent. Perfect 90-degree overhead angle, no perspective tilt.
+Objects fill approximately 70% of frame. Negative space is the green surface.
+MOOD:
+Clean, precise, performance-driven. Gym gear meets macro-perfect meal prep.
+CAMERA SYSTEM:
+Canon R5 / Sony A7R IV. Natural lens perspective equivalent to 35mm-50mm full-frame.
+No wide-angle distortion. No telephoto compression.
+CAMERA SETTINGS (product flat-lay):
+ISO 200. Shutter 1/160 sec. Aperture f/2.8. Color temperature 5200K, neutral white balance.
+LIGHTING:
+Natural daylight only. No artificial flash, no studio strobes, no colored gels.
+Shadows are crisp and clean. Highlights are clean, not blown.
+COLOR TREATMENT:
+True-to-life color. Neutral whites — no yellow, orange, or blue cast.
+Balanced contrast — never cinematic or overgraded. No LUTs. No filters. No stylization.
+TEXTURE REALISM:
+Product surfaces show material texture — frosted plastic lid, matte fabric weave, metal finish.
+DEPTH OF FIELD:
+All objects in sharp focus. Flat-lay — no depth blur.
+COMPOSITION:
+Intentional but unstyled. Everything feels observed, not staged.
+Clear product hierarchy. Use of negative space for premium, clean feel.
+No floating objects. All objects fully grounded with correct shadows.
+STRICT OUTPUT:
+No text overlays. No logos other than Delicut branding on product.
+No UI elements. No signage.
+Ultra-high-definition editorial realism. Natural grain, not noise-free plastic look.</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0318-0125_abstract-green_Flux1Pro.png</t>
+  </si>
+  <si>
+    <t>SCENE:
+Modern kitchen. Clean, minimal interior — white or light stone countertop visible.
+Refrigerator open in the background, interior light on. Time of day: morning.
+Natural light from a window to the left, soft and muted. Desaturated, cool-toned palette.
+SUBJECT:
+Athletic male, late 20s to early 30s. Lean but not bulky — fitness-conscious physique.
+Wearing a clean fitted white or grey t-shirt and training shorts.
+Natural, relaxed posture — not flexing, not posed.
+POSE:
+Reaching into the fridge or holding a Delicut meal prep container at chest height.
+Looking at the container with a natural satisfied expression — mid-moment, not smiling for camera.
+Weight shifted slightly to one leg. Arm extended naturally toward fridge.
+One hand holding the container only — correct finger count and natural grip.
+PRODUCT:
+Delicut meal prep container. Round shallow form factor, approximately 18cm diameter and 6cm tall.
+Deep spinach-green (#043F12) exterior sleeve printed with /delicut/ in bold white sans-serif lettering.
+Clear snap-on plastic lid with a silver rim edge.
+LID LABEL — CRITICAL RULES:
+The white square adhesive label (60x60mm) sits FLAT on the TOP of the lid — the horizontal top surface only.
+When the container is held at chest height and viewed from a 3/4 angle, the label is visible on TOP of the lid.
+The label NEVER appears sideways. The label NEVER wraps around the rim or side of the container.
+If the container side is in view, only the /delicut/ text on the green sleeve is visible — NOT the label.
+Label contents on top: /delicut/ logo | dish name | macro grid | customer name "Ahmed Al Mansoori"
+FOOD INSIDE:
+Visible through the clear lid when viewed from slightly above — grilled chicken breast,
+roasted broccoli and capsicum, a portion of fluffy quinoa. Vibrant, appetising colours.
+PRODUCT RULES:
+- Container exterior must be deep spinach-green (#043F12) — not beige, not red, not brown
+- /delicut/ branding in white, forward slashes, clearly readable on the green sleeve
+- Lid label flat on TOP of lid only — NEVER sideways, NEVER on the side
+- Do not alter, recolor, or redesign any element
+LIGHTING:
+Soft, minimal, desaturated morning light from left window. Muted diffused quality.
+Fridge interior light adds very subtle warm fill from behind. No flash. No overhead spot.
+Minimal shadows — soft falloff only, no hard shadow edges. 5600K neutral white.
+CAMERA:
+35mm equivalent. Eye-level, slightly elevated angle.
+Three-quarter body shot — top of head to mid-thigh. Subject slightly left of center.
+Background kitchen and open fridge softly out of focus but readable.
+Use lifestyle/action camera settings.
+MOOD:
+Effortless healthy living. The fridge-smile moment — satisfaction without effort.
+Desaturated palette — muted, calm, editorial feel. Not vibrant or oversaturated.
+CAMERA SYSTEM:
+Canon R5 / Sony A7R IV. Natural lens perspective equivalent to 35mm-50mm full-frame.
+No wide-angle distortion. No telephoto compression.
+CAMERA SETTINGS (lifestyle / action):
+ISO 400. Shutter 1/1600 sec. Aperture f/4. Color temperature 5600K, neutral white balance.
+LIGHTING:
+Natural daylight only. No artificial flash, no studio strobes, no colored gels.
+Shadows are minimal and soft. Highlights are clean, not blown.
+COLOR TREATMENT:
+Desaturated, muted color grading. Neutral whites — no yellow, orange, or blue cast.
+Low contrast — never cinematic or overgraded. No LUTs. No filters. Calm editorial look.
+TEXTURE REALISM:
+Visible skin texture — natural pores, no sweat.
+Fabric shows natural behavior — wrinkles, stretch, folds at joints.
+Product surfaces show material texture — clear plastic lid, matte plastic exterior.
+DEPTH OF FIELD:
+Subject or hero product in sharp focus. Background softly blurred but contextually readable.
+COMPOSITION:
+Intentional but unstyled. Everything feels observed, not staged.
+Clear subject hierarchy. Use of negative space for premium, clean feel.
+No floating objects. Correct gravity, minimal shadows, soft light falloff.
+STRICT OUTPUT:
+No text overlays. No logos other than Delicut branding on product.
+No UI elements. No signage. Correct human anatomy and natural proportions.
+Ultra-high-definition editorial realism. Natural grain, not noise-free plastic look.</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0318-0125_fridge-moment_Flux1Pro.png</t>
+  </si>
+  <si>
+    <t>SCENE:
+Gym locker room or quiet gym corner. Wooden bench in foreground.
+Lockers or a plain gym wall softly out of focus in background.
+Subdued, post-workout atmosphere — natural light from a high side window.
+SUBJECT:
+Athletic male, 28-32. Lean defined physique — not bulky, functionally fit.
+Wearing dark fitted compression shorts and a sleeveless training top.
+Natural post-workout state: slightly flushed, light sweat on arms and neck.
+POSE:
+Sitting on the bench. Forearms resting on knees, slight forward lean.
+Head slightly down, composed and focused — the stillness after a hard session.
+Not looking at camera. Hands relaxed, fingers loosely interlaced. Correct finger count.
+PRODUCT — SIZE IS CRITICAL:
+Delicut meal prep container placed on the bench beside the seated male.
+Container diameter is approximately 18cm and 8cm tall — roughly the size of a dinner plate.
+This is a realistic food storage container — NOT a tiny snack box, NOT oversized.
+It should look proportionally correct next to a seated adult male's body.
+Container: Round shallow form factor. Deep spinach-green (#043F12) exterior sleeve.
+The word /delicut/ appears in ONE single horizontal line in bold white sans-serif on the side of the sleeve.
+Do NOT repeat the text multiple times. ONE clear instance of /delicut/ in a single line.
+Clear snap-on plastic lid with a silver rim edge.
+LID LABEL — CRITICAL RULES:
+A white square adhesive label (60x60mm) sits FLAT on the TOP of the lid — horizontal top surface only.
+The label is NEVER on the side of the container. NEVER sideways. NEVER on the rim.
+Label contents:
+- /delicut/ logo in bold sans-serif
+- Dish name: "Grilled Chicken &amp; Roasted Vegetables"
+- Macro grid: kcal 480 | pro 42g | carbs 28g | fat 14g
+- Customer name: "Ahmed Al Mansoori" clearly printed at the bottom of the label
+FOOD INSIDE:
+Visible through the clear lid — grilled chicken breast sliced on the diagonal,
+roasted broccoli and capsicum, a portion of fluffy quinoa. Vibrant, appetising colours.
+Moisture on the vegetables catching light.
+PRODUCT RULES:
+- Container exterior must be deep spinach-green (#043F12) — not beige, not red, not brown
+- /delicut/ in ONE single horizontal line in white — not repeated, not wrapped
+- Container scale: ~18cm diameter, ~8cm tall — realistic relative to seated adult male
+- Lid label flat on top only — NEVER sideways
+- Do not alter, recolor, or redesign any element
+LIGHTING:
+Natural side light from a high window. Single light source, slightly directional.
+Soft shadows across the locker room floor. Highlights on tray lid and subject's arms.
+No artificial fill. No rim light. 5600K neutral white.
+CAMERA:
+35mm equivalent. Low to mid angle — camera slightly below bench height.
+Focus on tray (sharp). Subject mid-ground, slightly blurred (depth of field).
+Mid-shot — bench surface to subject's shoulders. Tray occupies left third of frame.
+Use lifestyle/action camera settings.
+MOOD:
+Disciplined. Post-effort calm. The meal is the reward.
+CAMERA SYSTEM:
+Canon R5 / Sony A7R IV. Natural lens perspective equivalent to 35mm-50mm full-frame.
+No wide-angle distortion. No telephoto compression.
+CAMERA SETTINGS (lifestyle / action):
+ISO 400. Shutter 1/1600 sec. Aperture f/4. Color temperature 5600K, neutral white balance.
+LIGHTING:
+Natural daylight only. No artificial flash, no studio strobes, no colored gels.
+Shadows are soft falloff. Highlights are clean, not blown.
+COLOR TREATMENT:
+True-to-life color. Neutral whites — no yellow, orange, or blue cast.
+Balanced contrast — never cinematic or overgraded. No LUTs. No filters. No stylization.
+TEXTURE REALISM:
+Visible skin texture — natural pores, light sweat sheen where appropriate.
+Fabric shows natural behavior — wrinkles, stretch, folds at joints.
+Product surfaces show material texture — matte plastic, clear lid.
+DEPTH OF FIELD:
+Product in sharp focus. Subject mid-ground softly blurred but face readable.
+COMPOSITION:
+Intentional but unstyled. Everything feels observed, not staged.
+Clear subject hierarchy. Use of negative space for premium, clean feel.
+No floating objects. Correct gravity, shadows, and light falloff.
+STRICT OUTPUT:
+No text overlays. No logos other than Delicut branding on product.
+No UI elements. No signage. Correct human anatomy and natural proportions.
+Ultra-high-definition editorial realism. Natural grain, not noise-free plastic look.</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0318-0125_post-workout-bench_Flux1Pro.png</t>
+  </si>
+  <si>
+    <t>no delicut box generated</t>
+  </si>
+  <si>
+    <t>human antomy very incorrect. Delicut box is rendered as a single green box. Delicut logo not seen. Human is holding the box from the side instead of on the palm</t>
+  </si>
+  <si>
+    <t>reject. No product image seen. Only a bulked up man without any photo realistic features</t>
   </si>
 </sst>
 </file>
@@ -829,7 +1651,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="6" width="22" customWidth="1"/>
@@ -1223,7 +2045,7 @@
         <v>35</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="316.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1249,13 +2071,13 @@
         <v>24</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I13" s="2">
         <v>1</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="K13" s="2" t="s">
         <v>18</v>
@@ -1263,7 +2085,7 @@
     </row>
     <row r="14" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>12</v>
@@ -1281,16 +2103,16 @@
         <v>15</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I14" s="2">
         <v>1</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>18</v>
@@ -1298,7 +2120,7 @@
     </row>
     <row r="15" spans="1:11" ht="316.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>12</v>
@@ -1316,16 +2138,16 @@
         <v>15</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="I15" s="2">
         <v>1</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K15" s="2" t="s">
         <v>18</v>
@@ -1333,7 +2155,7 @@
     </row>
     <row r="16" spans="1:11" ht="345.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>12</v>
@@ -1351,24 +2173,24 @@
         <v>15</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I16" s="2">
         <v>5</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="345.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>12</v>
@@ -1398,7 +2220,7 @@
         <v>51</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1541,7 +2363,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>63</v>
       </c>
@@ -1568,13 +2390,13 @@
       </c>
       <c r="I22" s="2"/>
       <c r="J22" s="2" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="K22" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>63</v>
       </c>
@@ -1601,13 +2423,13 @@
       </c>
       <c r="I23" s="2"/>
       <c r="J23" s="2" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="K23" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>63</v>
       </c>
@@ -1634,13 +2456,13 @@
       </c>
       <c r="I24" s="2"/>
       <c r="J24" s="2" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="K24" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>63</v>
       </c>
@@ -1667,15 +2489,15 @@
       </c>
       <c r="I25" s="2"/>
       <c r="J25" s="2" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="K25" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>12</v>
@@ -1696,19 +2518,19 @@
         <v>53</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I26" s="2"/>
       <c r="J26" s="2" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="K26" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>12</v>
@@ -1729,19 +2551,19 @@
         <v>56</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I27" s="2"/>
       <c r="J27" s="2" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="K27" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>12</v>
@@ -1762,19 +2584,19 @@
         <v>59</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I28" s="2"/>
       <c r="J28" s="2" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="K28" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>12</v>
@@ -1795,19 +2617,19 @@
         <v>61</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I29" s="2"/>
       <c r="J29" s="2" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="K29" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>12</v>
@@ -1828,21 +2650,21 @@
         <v>53</v>
       </c>
       <c r="H30" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="I30" s="2">
+        <v>1</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="I30" s="2">
-        <v>1</v>
-      </c>
-      <c r="J30" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="K30" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="2" t="s">
-        <v>68</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>12</v>
@@ -1863,21 +2685,21 @@
         <v>56</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I31" s="2">
         <v>1</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K31" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>12</v>
@@ -1898,21 +2720,21 @@
         <v>59</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="I32" s="2">
         <v>1</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K32" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>12</v>
@@ -1933,7 +2755,7 @@
         <v>61</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="I33" s="2">
         <v>1</v>
@@ -1942,6 +2764,426 @@
         <v>77</v>
       </c>
       <c r="K33" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C34" s="2">
+        <v>5</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="I34" s="2">
+        <v>1</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C35" s="2">
+        <v>5</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="I35" s="2">
+        <v>1</v>
+      </c>
+      <c r="J35" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="K35" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C36" s="2">
+        <v>5</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="I36" s="2">
+        <v>2</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C37" s="2">
+        <v>5</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="I37" s="2">
+        <v>2</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C38" s="2">
+        <v>6</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="I38" s="2">
+        <v>1</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C39" s="2">
+        <v>6</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="I39" s="2">
+        <v>1</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C40" s="2">
+        <v>6</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="I40" s="2">
+        <v>1</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C41" s="2">
+        <v>6</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="I41" s="2">
+        <v>1</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C42" s="2">
+        <v>7</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="I42" s="2">
+        <v>1</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A43" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C43" s="2">
+        <v>7</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="I43" s="2">
+        <v>1</v>
+      </c>
+      <c r="J43" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="K43" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C44" s="2">
+        <v>7</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="I44" s="2">
+        <v>1</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C45" s="2">
+        <v>7</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="I45" s="2">
+        <v>1</v>
+      </c>
+      <c r="J45" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="K45" s="2" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feedback on stable diffusion with changes to prompt
</commit_message>
<xml_diff>
--- a/outputs/session_log.xlsx
+++ b/outputs/session_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ramakant\VSCode-projects\delicut-creative-workflow\outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EA3ABFB-DA52-4B5C-A6EA-016FA2C71BE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45C84DF0-1684-4302-9986-9E8133DFD3DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="131">
   <si>
     <t>session_id</t>
   </si>
@@ -1135,6 +1135,9 @@
     <t>outputs\images\harry_0318-0125_abstract-green_Flux1Pro.png</t>
   </si>
   <si>
+    <t>no delicut box generated</t>
+  </si>
+  <si>
     <t>SCENE:
 Modern kitchen. Clean, minimal interior — white or light stone countertop visible.
 Refrigerator open in the background, interior light on. Time of day: morning.
@@ -1206,6 +1209,9 @@
   </si>
   <si>
     <t>outputs\images\harry_0318-0125_fridge-moment_Flux1Pro.png</t>
+  </si>
+  <si>
+    <t>human antomy very incorrect. Delicut box is rendered as a single green box. Delicut logo not seen. Human is holding the box from the side instead of on the palm</t>
   </si>
   <si>
     <t>SCENE:
@@ -1288,13 +1294,49 @@
     <t>outputs\images\harry_0318-0125_post-workout-bench_Flux1Pro.png</t>
   </si>
   <si>
-    <t>no delicut box generated</t>
-  </si>
-  <si>
-    <t>human antomy very incorrect. Delicut box is rendered as a single green box. Delicut logo not seen. Human is holding the box from the side instead of on the palm</t>
-  </si>
-  <si>
     <t>reject. No product image seen. Only a bulked up man without any photo realistic features</t>
+  </si>
+  <si>
+    <t>harry_0318-0133</t>
+  </si>
+  <si>
+    <t>SD35Large</t>
+  </si>
+  <si>
+    <t>ERROR: 402 Client Error: Payment Required for url: https://api.replicate.com/v1/models/stability-ai/stable-diffusion-3.5-large/predictions</t>
+  </si>
+  <si>
+    <t>harry_0318-0136</t>
+  </si>
+  <si>
+    <t>harry_0318-0138</t>
+  </si>
+  <si>
+    <t>harry_0318-0139</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0318-0139_treadmill-female_SD35Large.png</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0318-0139_abstract-green_SD35Large.png</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0318-0139_fridge-moment_SD35Large.png</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0318-0139_post-workout-bench_SD35Large.png</t>
+  </si>
+  <si>
+    <t>anatomy is correct but she's running sideways perpendicular to the treadmill. This is AI slop</t>
+  </si>
+  <si>
+    <t>no product shown only black box rendered</t>
+  </si>
+  <si>
+    <t>human is holding steel pan instead of delicut meal box. Anatomy is not photo-realistic</t>
+  </si>
+  <si>
+    <t>delicut meal box is not in the image. Anatomy is not life-like with bulging shoulders and not photorealistic</t>
   </si>
 </sst>
 </file>
@@ -1651,7 +1693,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K45"/>
+  <dimension ref="A1:K59"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="6" width="22" customWidth="1"/>
@@ -3047,7 +3089,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>104</v>
       </c>
@@ -3082,7 +3124,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>104</v>
       </c>
@@ -3111,13 +3153,13 @@
         <v>1</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="K43" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>104</v>
       </c>
@@ -3137,22 +3179,22 @@
         <v>15</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I44" s="2">
         <v>1</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="K44" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>104</v>
       </c>
@@ -3172,10 +3214,10 @@
         <v>15</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="I45" s="2">
         <v>1</v>
@@ -3184,6 +3226,456 @@
         <v>116</v>
       </c>
       <c r="K45" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C46" s="2">
+        <v>8</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="I46" s="2"/>
+      <c r="J46" s="2"/>
+      <c r="K46" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A47" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C47" s="2">
+        <v>8</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="I47" s="2"/>
+      <c r="J47" s="2"/>
+      <c r="K47" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A48" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C48" s="2">
+        <v>8</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="I48" s="2"/>
+      <c r="J48" s="2"/>
+      <c r="K48" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A49" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C49" s="2">
+        <v>8</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="I49" s="2"/>
+      <c r="J49" s="2"/>
+      <c r="K49" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A50" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C50" s="2">
+        <v>9</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="I50" s="2"/>
+      <c r="J50" s="2"/>
+      <c r="K50" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A51" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C51" s="2">
+        <v>9</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="I51" s="2"/>
+      <c r="J51" s="2"/>
+      <c r="K51" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A52" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C52" s="2">
+        <v>9</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="H52" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="I52" s="2"/>
+      <c r="J52" s="2"/>
+      <c r="K52" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A53" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C53" s="2">
+        <v>9</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="I53" s="2"/>
+      <c r="J53" s="2"/>
+      <c r="K53" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A54" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C54" s="2">
+        <v>10</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="H54" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="I54" s="2"/>
+      <c r="J54" s="2"/>
+      <c r="K54" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A55" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C55" s="2">
+        <v>10</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="I55" s="2"/>
+      <c r="J55" s="2"/>
+      <c r="K55" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A56" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C56" s="2">
+        <v>11</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="I56" s="2">
+        <v>1</v>
+      </c>
+      <c r="J56" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="K56" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A57" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C57" s="2">
+        <v>11</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="I57" s="2">
+        <v>1</v>
+      </c>
+      <c r="J57" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="K57" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A58" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C58" s="2">
+        <v>11</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="H58" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="I58" s="2">
+        <v>1</v>
+      </c>
+      <c r="J58" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="K58" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A59" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C59" s="2">
+        <v>11</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H59" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="I59" s="2">
+        <v>1</v>
+      </c>
+      <c r="J59" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="K59" s="2" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
created gemini py file
</commit_message>
<xml_diff>
--- a/outputs/session_log.xlsx
+++ b/outputs/session_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ramakant\VSCode-projects\delicut-creative-workflow\outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45C84DF0-1684-4302-9986-9E8133DFD3DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1235743E-62AA-463B-A440-3160DDD7083D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="551" uniqueCount="144">
   <si>
     <t>session_id</t>
   </si>
@@ -1318,25 +1318,132 @@
     <t>outputs\images\harry_0318-0139_treadmill-female_SD35Large.png</t>
   </si>
   <si>
+    <t>anatomy is correct but she's running sideways perpendicular to the treadmill. This is AI slop</t>
+  </si>
+  <si>
     <t>outputs\images\harry_0318-0139_abstract-green_SD35Large.png</t>
   </si>
   <si>
+    <t>no product shown only black box rendered</t>
+  </si>
+  <si>
     <t>outputs\images\harry_0318-0139_fridge-moment_SD35Large.png</t>
   </si>
   <si>
+    <t>human is holding steel pan instead of delicut meal box. Anatomy is not photo-realistic</t>
+  </si>
+  <si>
     <t>outputs\images\harry_0318-0139_post-workout-bench_SD35Large.png</t>
   </si>
   <si>
-    <t>anatomy is correct but she's running sideways perpendicular to the treadmill. This is AI slop</t>
-  </si>
-  <si>
-    <t>no product shown only black box rendered</t>
-  </si>
-  <si>
-    <t>human is holding steel pan instead of delicut meal box. Anatomy is not photo-realistic</t>
-  </si>
-  <si>
     <t>delicut meal box is not in the image. Anatomy is not life-like with bulging shoulders and not photorealistic</t>
+  </si>
+  <si>
+    <t>harry_0318-0150</t>
+  </si>
+  <si>
+    <t>Photorealistic DSLR photograph. A lean athletic woman in her mid-20s running on a treadmill in a modern gym.
+CRITICAL — RUNNING DIRECTION:
+She is running ALONG the length of the treadmill belt. Her entire body faces directly toward the camera. Her left and right feet move FORWARD and BACKWARD along the treadmill belt. She is absolutely NOT running sideways. She is NOT perpendicular to the treadmill. She faces the camera head-on as if the camera is placed directly in front of the treadmill.
+SUBJECT:
+Lean athletic female, mid-20s. Toned physique, natural proportions, not bodybuilder.
+Fitted sports bra and high-waist training shorts. Hair in high ponytail. Light sweat sheen on skin.
+Mid-stride, one foot forward, one foot back, leaning slightly forward. Strong forward gaze.
+SCENE:
+Modern commercial gym. Rows of treadmills behind her. Mirrors on the wall. Natural light from large windows on the left. Background softly blurred.
+NO PRODUCT. No containers, no food, no packaging of any kind.
+CAMERA: Canon R5, 50mm lens, eye-level, mid-thigh to head crop, f/4, ISO 400, 1/1600s shutter, 5600K.
+Natural daylight only. Soft diffused light from left. No flash.
+True-to-life color, balanced contrast, no filters.
+Ultra-high-definition photorealistic image, natural skin texture, correct human anatomy.</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0318-0150_treadmill-female_SD35Large.png</t>
+  </si>
+  <si>
+    <t>Photorealistic overhead flat-lay product photograph shot on Canon R5, 50mm lens, 90-degree top-down angle.
+SURFACE: Dark forest green background, deep spinach green color.
+HERO PRODUCT — center of frame:
+A round circular plastic meal prep food container, approximately 18cm diameter and 6cm tall.
+The exterior sides are dark green plastic with white text on the side.
+The lid is a slightly frosted/translucent circular plastic lid with a silver rim.
+A small white rectangular paper label is stuck flat on the center top of the lid.
+The label has small black printed text showing a meal name and nutrition information.
+Inside the container, visible through the frosted lid: grilled chicken, broccoli, and quinoa.
+NO black borders on the container. NOT a black box. NOT an opaque black cube.
+SURROUNDING OBJECTS on the green surface:
+- A white chalk-dusted weight plate at upper-left
+- A folded white gym towel at lower-right
+- A silver stainless steel water bottle at lower-left
+Each object casts a soft shadow on the green surface.
+CAMERA: Perfect 90-degree overhead, f/2.8, ISO 200, 1/160s, 5200K.
+Hard directional overhead studio light. Crisp clean shadows. No colored gels.
+All objects in sharp focus. True-to-life color, no filters.
+Ultra-high-definition product photography realism.</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0318-0150_abstract-green_SD35Large.png</t>
+  </si>
+  <si>
+    <t>Photorealistic DSLR lifestyle photograph. A lean athletic man in his late 20s standing in a modern kitchen, reaching into an open refrigerator.
+SUBJECT:
+Athletic male, late 20s, lean natural physique — not bulky, not a bodybuilder, normal fit person.
+Wearing a fitted grey t-shirt and training shorts. Relaxed natural posture.
+Looking at what he is holding with a calm satisfied expression. NOT posing for the camera.
+Correct human anatomy — natural hands, correct number of fingers, realistic proportions.
+WHAT HE IS HOLDING:
+A round circular plastic food storage container, approximately 18cm wide.
+The container has a dark green plastic exterior and a clear plastic snap-on lid.
+NOT a pan. NOT a pot. NOT a steel pan. NOT cookware. NOT metallic cookware.
+This is a plastic meal prep container — like a round takeaway food box with a clear lid.
+He holds it flat on his palm at chest height, lid facing up toward camera.
+SCENE:
+Modern minimal kitchen. White or light stone countertop. Open refrigerator in background with interior light on.
+Natural morning light from window on the left. Background softly out of focus.
+CAMERA: Canon R5, 35mm lens, eye-level angle, three-quarter body shot (head to mid-thigh), f/4, ISO 400, 5600K.
+Soft diffused natural light. Muted, desaturated tones. Minimal shadows.
+True-to-life color, no filters, no oversaturation.
+Ultra-high-definition photorealistic image, correct human anatomy, natural skin texture.</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0318-0150_fridge-moment_SD35Large.png</t>
+  </si>
+  <si>
+    <t>Photorealistic DSLR lifestyle photograph. A lean athletic man sitting on a wooden bench in a gym locker room, with a green meal prep container placed on the bench beside him.
+SUBJECT:
+Athletic male, 28-32. Lean natural physique — toned but NOT a bodybuilder, NO exaggerated or bulging muscles.
+Normal fit person with natural shoulder width. Wearing compression shorts and a sleeveless training top.
+Sitting on bench, forearms resting on knees, slight forward lean, head slightly down.
+Post-workout calm. Not looking at camera. Natural relaxed hands, correct finger count.
+PRODUCT — MUST BE IN THE IMAGE:
+A round circular plastic food container sitting on the wooden bench to his left side, in sharp focus.
+The container is approximately 18cm wide and 8cm tall — about the size of a dinner plate, proportionally correct next to a seated adult.
+The container has a dark green plastic exterior and a clear plastic snap-on lid with a silver rim.
+A small white rectangular label is stuck on top of the lid with small black printed text.
+This container is clearly visible and prominent in the foreground of the image.
+NOT a tiny box. NOT absent from the image. It MUST appear beside him on the bench.
+SCENE:
+Gym locker room or gym corner. Wooden bench. Lockers or plain wall softly out of focus in background.
+Subdued post-workout atmosphere. Natural side light from a high window.
+CAMERA: Canon R5, 35mm lens, slightly below bench height, mid-shot (bench to shoulders), f/4, ISO 400, 5600K.
+Product in sharp focus, subject slightly blurred. Natural side light, soft shadows.
+True-to-life color, no filters, balanced contrast.
+Ultra-high-definition photorealistic image, correct human anatomy, natural proportions.</t>
+  </si>
+  <si>
+    <t>outputs\images\harry_0318-0150_post-workout-bench_SD35Large.png</t>
+  </si>
+  <si>
+    <t>female anatomy is ok. But the treadmilll is not rendered correctly. No rows of treadmills seen. She is not facing the camera as per the prompt instead camera is behind her. Photo realistic effect is missing</t>
+  </si>
+  <si>
+    <t>no surrounding objects. No hero product shown. A black round box is seen which is not as per prompt</t>
+  </si>
+  <si>
+    <t>human anatomy is all incorrect. The elbows are bulging with veins shown. This is not realistic at all. Shirt on right shoulder is not rendered correctly.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">photo realism , human and setting is correct. But no product image is seen. </t>
   </si>
 </sst>
 </file>
@@ -1693,7 +1800,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K59"/>
+  <dimension ref="A1:K63"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="6" width="22" customWidth="1"/>
@@ -3229,7 +3336,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>117</v>
       </c>
@@ -3260,7 +3367,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>117</v>
       </c>
@@ -3291,7 +3398,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>117</v>
       </c>
@@ -3322,7 +3429,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>117</v>
       </c>
@@ -3353,7 +3460,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>120</v>
       </c>
@@ -3384,7 +3491,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>120</v>
       </c>
@@ -3415,7 +3522,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>120</v>
       </c>
@@ -3446,7 +3553,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>120</v>
       </c>
@@ -3477,7 +3584,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="54" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>121</v>
       </c>
@@ -3508,7 +3615,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="55" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>121</v>
       </c>
@@ -3539,7 +3646,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="56" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>122</v>
       </c>
@@ -3568,13 +3675,13 @@
         <v>1</v>
       </c>
       <c r="J56" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="K56" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="57" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>122</v>
       </c>
@@ -3597,19 +3704,19 @@
         <v>108</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I57" s="2">
         <v>1</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="K57" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="58" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>122</v>
       </c>
@@ -3632,19 +3739,19 @@
         <v>111</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I58" s="2">
         <v>1</v>
       </c>
       <c r="J58" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K58" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="59" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:11" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>122</v>
       </c>
@@ -3667,7 +3774,7 @@
         <v>114</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="I59" s="2">
         <v>1</v>
@@ -3676,6 +3783,146 @@
         <v>130</v>
       </c>
       <c r="K59" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A60" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C60" s="2">
+        <v>12</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="I60" s="2">
+        <v>2</v>
+      </c>
+      <c r="J60" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="K60" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A61" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C61" s="2">
+        <v>12</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="H61" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="I61" s="2">
+        <v>1</v>
+      </c>
+      <c r="J61" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="K61" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A62" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C62" s="2">
+        <v>12</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="H62" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="I62" s="2">
+        <v>1</v>
+      </c>
+      <c r="J62" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="K62" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A63" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C63" s="2">
+        <v>12</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="H63" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="I63" s="2">
+        <v>2</v>
+      </c>
+      <c r="J63" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="K63" s="2" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
scripts and prompts updated with more ref images
</commit_message>
<xml_diff>
--- a/outputs/session_log.xlsx
+++ b/outputs/session_log.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K71"/>
+  <dimension ref="A1:K83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="6"/>
@@ -6505,7 +6505,7 @@
         </is>
       </c>
     </row>
-    <row r="68">
+    <row r="68" ht="409.6" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
           <t>harry_0318-0221</t>
@@ -6562,15 +6562,21 @@
           <t>ERROR: 422 Client Error: Unprocessable Entity for url: https://fal.run/fal-ai/bria/product-shot</t>
         </is>
       </c>
-      <c r="I68" s="2" t="inlineStr"/>
-      <c r="J68" s="2" t="inlineStr"/>
+      <c r="I68" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
+          <t>reject</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="409.6" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
         <is>
           <t>harry_0318-0221</t>
@@ -6633,15 +6639,21 @@
           <t>ERROR: 422 Client Error: Unprocessable Entity for url: https://fal.run/fal-ai/bria/product-shot</t>
         </is>
       </c>
-      <c r="I69" s="2" t="inlineStr"/>
-      <c r="J69" s="2" t="inlineStr"/>
+      <c r="I69" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
+          <t>reject</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="409.6" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
           <t>harry_0318-0221</t>
@@ -6701,15 +6713,21 @@
           <t>ERROR: 422 Client Error: Unprocessable Entity for url: https://fal.run/fal-ai/bria/product-shot</t>
         </is>
       </c>
-      <c r="I70" s="2" t="inlineStr"/>
-      <c r="J70" s="2" t="inlineStr"/>
+      <c r="I70" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
+          <t>reject</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="409.6" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
           <t>harry_0318-0221</t>
@@ -6766,9 +6784,846 @@
           <t>ERROR: 422 Client Error: Unprocessable Entity for url: https://fal.run/fal-ai/bria/product-shot</t>
         </is>
       </c>
-      <c r="I71" s="2" t="inlineStr"/>
-      <c r="J71" s="2" t="inlineStr"/>
+      <c r="I71" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
       <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>reject</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="409.6" customHeight="1">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>harry_0318-0223</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>healthy-harry</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>BriaProductShot</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>1080x1080</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Photorealistic DSLR photograph. A lean athletic woman in her mid-20s running on a treadmill in a modern gym.
+CAMERA POSITION AND RUNNING DIRECTION — CRITICAL:
+The camera is placed DIRECTLY IN FRONT of the treadmill, at eye level, facing the runner head-on.
+The woman runs STRAIGHT TOWARD the camera — like a runner approaching the finish line.
+From the camera's perspective she moves closer, not left or right.
+Her feet alternate forward and backward along the treadmill belt — one foot strikes in front, one pushes behind.
+She is NOT running sideways. She is NOT perpendicular to the treadmill. She does NOT face left or right.
+Rows of treadmills are visible BEHIND HER receding into the background.
+SUBJECT:
+Lean athletic female, mid-20s. Toned physique, natural proportions, not bodybuilder.
+Fitted sports bra and high-waist training shorts. Hair in high ponytail. Light sweat sheen on skin.
+Mid-stride, slight forward lean, strong gaze directly into the lens.
+SCENE:
+Modern commercial gym. Multiple rows of treadmills receding behind her. Mirrors on the wall reflecting gym interior. Natural light from large windows on the left. Background softly blurred.
+NO PRODUCT. No containers, no food, no packaging of any kind.
+CAMERA: Canon R5, 50mm lens, eye-level directly in front of treadmill, mid-thigh to head crop, f/4, ISO 400, 1/1600s shutter, 5600K.
+Natural daylight only. Soft diffused light from left. No flash.
+True-to-life color, balanced contrast, no filters.
+Ultra-high-definition photorealistic image, natural skin texture, correct human anatomy.</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>outputs\images\harry_0318-0223_treadmill-female_BriaProductShot.png</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>there is no woman nor any treadmill</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>reject</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="409.6" customHeight="1">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>harry_0318-0223</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>healthy-harry</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>BriaProductShot</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>1080x1080</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Photorealistic overhead flat-lay product photograph shot on Canon R5, 50mm lens, 90-degree top-down angle.
+SURFACE: Deep spinach-green background, hex #043F12.
+HERO PRODUCT — centered in frame:
+A single round shallow plastic food container, compact and low-profile, approximately 18cm diameter.
+Exterior sleeve is dark spinach-green printed with '/delicut' in bold white sans-serif uppercase letters.
+Topped with a clear snap-on plastic lid with a raised ridge rim.
+LID LABEL — flat on top of lid, square white adhesive label:
+- Top line: '/delicut/' logo bold sans-serif | delicut.ae URL
+- Meal name in large bold text: 'Grilled Chicken and Roasted Vegetables'
+- Meal category: 'High Protein Main'
+- Macro grid: kcal 480 | pro 42g | carbs 28g | fat 14g
+- Customer name: 'Ahmed Al Mansoori' | best before date | barcode
+All label text is crisp black on white. Clean typographic layout. All text legible.
+FOOD INSIDE — fully contained within the tray, visible through the clear lid:
+Grilled chicken breast sliced on the diagonal, roasted broccoli and capsicum, fluffy quinoa.
+Vibrant colours. Nothing spills outside the rim.
+SURROUNDING OBJECTS on the green surface:
+- A white chalk-dusted weight plate at upper-left
+- A folded white gym towel at lower-right
+- A matte stainless steel water bottle at lower-left
+Each object naturally grounded with a crisp shadow beneath it.
+CAMERA: Perfect 90-degree overhead, f/2.8, ISO 200, 1/160s, 5200K.
+Hard directional overhead studio light. Crisp clean shadows. No colored gels.
+All objects in sharp focus. True-to-life color, no filters.
+Ultra-high-definition product photography realism.</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>outputs\images\harry_0318-0223_abstract-green_BriaProductShot.png</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>best product shot till date. should consider this model for abstract images and food ideas</t>
+        </is>
+      </c>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="409.6" customHeight="1">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>harry_0318-0223</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>healthy-harry</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>BriaProductShot</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>1080x1080</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Photorealistic DSLR lifestyle photograph. A lean athletic man in his late 20s standing in a modern kitchen, reaching into an open refrigerator.
+SUBJECT:
+Athletic male, late 20s, lean natural physique — not bulky, not a bodybuilder, normal fit person.
+Wearing a fitted grey t-shirt and training shorts. Relaxed natural posture.
+Looking at what he is holding with a calm satisfied expression. NOT posing for the camera.
+Correct human anatomy — natural hands, correct number of fingers, realistic proportions.
+WHAT HE IS HOLDING:
+A round shallow PLASTIC food container, approximately 18cm wide and 6cm tall — like a takeaway bowl.
+This is a ready-to-eat meal prep container made of plastic with a removable clear plastic snap-on lid, sealed on all sides.
+NOT a thermos. NOT a steel bottle. NOT a metal container. NOT a pan. NOT cookware. NOT a jar.
+It is a round, low-profile plastic bowl with a flat clear lid — the kind used for delivered ready meals.
+He holds it flat on his palm at chest height, lid facing up.
+REFRIGERATOR:
+Open fridge in the background with the interior light on.
+Fridge shelves are STOCKED with food — vegetables, bottles of juice, produce, other meal containers.
+Not empty. Fridge looks like a well-stocked household refrigerator.
+SCENE:
+Modern minimal kitchen. White or light stone countertop. Natural morning light from window on the left.
+Background softly out of focus.
+CAMERA: Canon R5, 35mm lens, eye-level, three-quarter body shot (head to mid-thigh), f/4, ISO 400, 5600K.
+Soft diffused natural light. Minimal shadows. True-to-life color, no filters.
+Ultra-high-definition photorealistic image, correct human anatomy, natural skin texture.</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>outputs\images\harry_0318-0223_fridge-moment_BriaProductShot.png</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>human anatomy is missing head and arms. Fridge is completely wrong. Only the product is seen correct</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>reject</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="409.6" customHeight="1">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>harry_0318-0223</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>healthy-harry</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>BriaProductShot</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>1080x1080</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>Photorealistic DSLR lifestyle photograph. A lean athletic man sitting on a wooden bench in a gym locker room, with a Delicut meal prep container placed on the bench beside him.
+SUBJECT:
+Athletic male, 28-32. Lean natural physique — toned but NOT a bodybuilder, NO exaggerated or bulging muscles.
+Normal fit person with natural shoulder width. Wearing compression shorts and a sleeveless training top.
+Sitting on bench, forearms resting on knees, slight forward lean, head slightly down.
+Post-workout calm. Not looking at camera. Natural relaxed hands, correct finger count.
+PRODUCT — MUST BE IN THE IMAGE, placed on the bench to his left, in sharp focus:
+A round shallow plastic food container — compact and low-profile, approximately 18cm diameter.
+Exterior sleeve is dark spinach-green (#043F12) printed with '/delicut' in bold white sans-serif uppercase letters.
+Topped with a clear snap-on plastic lid with a raised ridge rim. No silver rim. No metallic rim.
+A small white square adhesive label sits flat on the TOP of the lid showing meal name and nutrition info.
+This container is clearly visible and prominent in the foreground — NOT absent, NOT tiny, NOT incorrect color.
+SCENE:
+Gym locker room or gym corner. Wooden bench. Lockers or plain wall softly out of focus in background.
+Subdued post-workout atmosphere. Natural side light from a high window.
+CAMERA: Canon R5, 35mm lens, slightly below bench height, mid-shot (bench to shoulders), f/4, ISO 400, 5600K.
+Product in sharp focus, subject slightly blurred. Natural side light, soft shadows.
+True-to-life color, no filters, balanced contrast.
+Ultra-high-definition photorealistic image, correct human anatomy, natural proportions.</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>outputs\images\harry_0318-0223_post-workout-bench_BriaProductShot.png</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>human anatomy is wrong. Too bulked up with bulging veins. Product image is correct</t>
+        </is>
+      </c>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>reject</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>harry_0318-0246</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>healthy-harry</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>BriaProductShot</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>1080x1080</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>Photorealistic DSLR photograph. A lean athletic woman in her mid-20s running on a treadmill in a modern gym.
+CAMERA POSITION AND RUNNING DIRECTION — CRITICAL:
+The camera is placed DIRECTLY IN FRONT of the treadmill, at eye level, facing the runner head-on.
+The woman runs STRAIGHT TOWARD the camera — like a runner approaching the finish line.
+From the camera's perspective she moves closer, not left or right.
+Her feet alternate forward and backward along the treadmill belt — one foot strikes in front, one pushes behind.
+She is NOT running sideways. She is NOT perpendicular to the treadmill. She does NOT face left or right.
+Rows of treadmills are visible BEHIND HER receding into the background.
+SUBJECT:
+Lean athletic female, mid-20s. Toned physique, natural proportions, not bodybuilder.
+Fitted sports bra and high-waist training shorts. Hair in high ponytail. Light sweat sheen on skin.
+Mid-stride, slight forward lean, strong gaze directly into the lens.
+SCENE:
+Modern commercial gym. Multiple rows of treadmills receding behind her. Mirrors on the wall reflecting gym interior. Natural light from large windows on the left. Background softly blurred.
+NO PRODUCT. No containers, no food, no packaging of any kind.
+CAMERA: Canon R5, 50mm lens, eye-level directly in front of treadmill, mid-thigh to head crop, f/4, ISO 400, 1/1600s shutter, 5600K.
+Natural daylight only. Soft diffused light from left. No flash.
+True-to-life color, balanced contrast, no filters.
+Ultra-high-definition photorealistic image, natural skin texture, correct human anatomy.</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>outputs\images\harry_0318-0246_treadmill-female_BriaProductShot.png</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr"/>
+      <c r="J76" s="2" t="inlineStr"/>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>harry_0318-0246</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>healthy-harry</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>BriaProductShot</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>1080x1080</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>Photorealistic overhead flat-lay product photograph shot on Canon R5, 50mm lens, 90-degree top-down angle.
+SURFACE: Deep spinach-green background, hex #043F12.
+HERO PRODUCT — centered in frame:
+A single round shallow plastic food container, compact and low-profile, approximately 18cm diameter.
+Exterior sleeve is dark spinach-green printed with '/delicut' in bold white sans-serif uppercase letters.
+Topped with a clear snap-on plastic lid with a raised ridge rim.
+LID LABEL — flat on top of lid, square white adhesive label:
+- Top line: '/delicut/' logo bold sans-serif | delicut.ae URL
+- Meal name in large bold text: 'Grilled Chicken and Roasted Vegetables'
+- Meal category: 'High Protein Main'
+- Macro grid: kcal 480 | pro 42g | carbs 28g | fat 14g
+- Customer name: 'Ahmed Al Mansoori' | best before date | barcode
+All label text is crisp black on white. Clean typographic layout. All text legible.
+FOOD INSIDE — fully contained within the tray, visible through the clear lid:
+Grilled chicken breast sliced on the diagonal, roasted broccoli and capsicum, fluffy quinoa.
+Vibrant colours. Nothing spills outside the rim.
+SURROUNDING OBJECTS on the green surface:
+- A white chalk-dusted weight plate at upper-left
+- A folded white gym towel at lower-right
+- A matte stainless steel water bottle at lower-left
+Each object naturally grounded with a crisp shadow beneath it.
+CAMERA: Perfect 90-degree overhead, f/2.8, ISO 200, 1/160s, 5200K.
+Hard directional overhead studio light. Crisp clean shadows. No colored gels.
+All objects in sharp focus. True-to-life color, no filters.
+Ultra-high-definition product photography realism.</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>outputs\images\harry_0318-0246_abstract-green_BriaProductShot.png</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr"/>
+      <c r="J77" s="2" t="inlineStr"/>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>harry_0318-0246</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>healthy-harry</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>BriaProductShot</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>1080x1080</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>Photorealistic DSLR lifestyle photograph. A lean athletic man in his late 20s standing in a modern kitchen, reaching into an open refrigerator.
+SUBJECT:
+Athletic male, late 20s, lean natural physique — not bulky, not a bodybuilder, normal fit person.
+Wearing a fitted grey t-shirt and training shorts. Relaxed natural posture.
+Looking at what he is holding with a calm satisfied expression. NOT posing for the camera.
+Correct human anatomy — natural hands, correct number of fingers, realistic proportions.
+WHAT HE IS HOLDING:
+A round shallow PLASTIC food container, approximately 18cm wide and 6cm tall — like a takeaway bowl.
+This is a ready-to-eat meal prep container made of plastic with a removable clear plastic snap-on lid, sealed on all sides.
+NOT a thermos. NOT a steel bottle. NOT a metal container. NOT a pan. NOT cookware. NOT a jar.
+It is a round, low-profile plastic bowl with a flat clear lid — the kind used for delivered ready meals.
+He holds it flat on his palm at chest height, lid facing up.
+REFRIGERATOR:
+Open fridge in the background with the interior light on.
+Fridge shelves are STOCKED with food — vegetables, bottles of juice, produce, other meal containers.
+Not empty. Fridge looks like a well-stocked household refrigerator.
+SCENE:
+Modern minimal kitchen. White or light stone countertop. Natural morning light from window on the left.
+Background softly out of focus.
+CAMERA: Canon R5, 35mm lens, eye-level, three-quarter body shot (head to mid-thigh), f/4, ISO 400, 5600K.
+Soft diffused natural light. Minimal shadows. True-to-life color, no filters.
+Ultra-high-definition photorealistic image, correct human anatomy, natural skin texture.</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>outputs\images\harry_0318-0246_fridge-moment_BriaProductShot.png</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr"/>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>harry_0318-0246</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>healthy-harry</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>BriaProductShot</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>1080x1080</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>Photorealistic DSLR lifestyle photograph. A lean athletic man sitting on a wooden bench in a gym locker room, with a Delicut meal prep container placed on the bench beside him.
+SUBJECT:
+Athletic male, 28-32. Lean natural physique — toned but NOT a bodybuilder, NO exaggerated or bulging muscles.
+Normal fit person with natural shoulder width. Wearing compression shorts and a sleeveless training top.
+Sitting on bench, forearms resting on knees, slight forward lean, head slightly down.
+Post-workout calm. Not looking at camera. Natural relaxed hands, correct finger count.
+PRODUCT — MUST BE IN THE IMAGE, placed on the bench to his left, in sharp focus:
+A round shallow plastic food container — compact and low-profile, approximately 18cm diameter.
+Exterior sleeve is dark spinach-green (#043F12) printed with '/delicut' in bold white sans-serif uppercase letters.
+Topped with a clear snap-on plastic lid with a raised ridge rim. No silver rim. No metallic rim.
+A small white square adhesive label sits flat on the TOP of the lid showing meal name and nutrition info.
+This container is clearly visible and prominent in the foreground — NOT absent, NOT tiny, NOT incorrect color.
+SCENE:
+Gym locker room or gym corner. Wooden bench. Lockers or plain wall softly out of focus in background.
+Subdued post-workout atmosphere. Natural side light from a high window.
+CAMERA: Canon R5, 35mm lens, slightly below bench height, mid-shot (bench to shoulders), f/4, ISO 400, 5600K.
+Product in sharp focus, subject slightly blurred. Natural side light, soft shadows.
+True-to-life color, no filters, balanced contrast.
+Ultra-high-definition photorealistic image, correct human anatomy, natural proportions.</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>outputs\images\harry_0318-0246_post-workout-bench_BriaProductShot.png</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr"/>
+      <c r="J79" s="2" t="inlineStr"/>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>harry_0318-0249</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>healthy-harry</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>Imagen4Ultra</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>1080x1080</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>Photorealistic DSLR photograph. A lean athletic woman in her mid-20s running on a treadmill in a modern gym.
+CAMERA POSITION AND RUNNING DIRECTION — CRITICAL:
+The camera is placed DIRECTLY IN FRONT of the treadmill, at eye level, facing the runner head-on.
+The woman runs STRAIGHT TOWARD the camera — like a runner approaching the finish line.
+From the camera's perspective she moves closer, not left or right.
+Her feet alternate forward and backward along the treadmill belt — one foot strikes in front, one pushes behind.
+She is NOT running sideways. She is NOT perpendicular to the treadmill. She does NOT face left or right.
+Rows of treadmills are visible BEHIND HER receding into the background.
+SUBJECT:
+Lean athletic female, mid-20s. Toned physique, natural proportions, not bodybuilder.
+Fitted sports bra and high-waist training shorts. Hair in high ponytail. Light sweat sheen on skin.
+Mid-stride, slight forward lean, strong gaze directly into the lens.
+SCENE:
+Modern commercial gym. Multiple rows of treadmills receding behind her. Mirrors on the wall reflecting gym interior. Natural light from large windows on the left. Background softly blurred.
+NO PRODUCT. No containers, no food, no packaging of any kind.
+CAMERA: Canon R5, 50mm lens, eye-level directly in front of treadmill, mid-thigh to head crop, f/4, ISO 400, 1/1600s shutter, 5600K.
+Natural daylight only. Soft diffused light from left. No flash.
+True-to-life color, balanced contrast, no filters.
+Ultra-high-definition photorealistic image, natural skin texture, correct human anatomy.</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>outputs\images\harry_0318-0249_treadmill-female_Imagen4Ultra.png</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr"/>
+      <c r="J80" s="2" t="inlineStr"/>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>harry_0318-0249</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>healthy-harry</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>Imagen4Ultra</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>1080x1080</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>Photorealistic overhead flat-lay product photograph shot on Canon R5, 50mm lens, 90-degree top-down angle.
+SURFACE: Deep spinach-green background, hex #043F12.
+HERO PRODUCT — centered in frame:
+A single round shallow plastic food container, compact and low-profile, approximately 18cm diameter.
+Exterior sleeve is dark spinach-green printed with '/delicut' in bold white sans-serif uppercase letters.
+Topped with a clear snap-on plastic lid with a raised ridge rim.
+LID LABEL — flat on top of lid, square white adhesive label:
+- Top line: '/delicut/' logo bold sans-serif | delicut.ae URL
+- Meal name in large bold text: 'Grilled Chicken and Roasted Vegetables'
+- Meal category: 'High Protein Main'
+- Macro grid: kcal 480 | pro 42g | carbs 28g | fat 14g
+- Customer name: 'Ahmed Al Mansoori' | best before date | barcode
+All label text is crisp black on white. Clean typographic layout. All text legible.
+FOOD INSIDE — fully contained within the tray, visible through the clear lid:
+Grilled chicken breast sliced on the diagonal, roasted broccoli and capsicum, fluffy quinoa.
+Vibrant colours. Nothing spills outside the rim.
+SURROUNDING OBJECTS on the green surface:
+- A white chalk-dusted weight plate at upper-left
+- A folded white gym towel at lower-right
+- A matte stainless steel water bottle at lower-left
+Each object naturally grounded with a crisp shadow beneath it.
+CAMERA: Perfect 90-degree overhead, f/2.8, ISO 200, 1/160s, 5200K.
+Hard directional overhead studio light. Crisp clean shadows. No colored gels.
+All objects in sharp focus. True-to-life color, no filters.
+Ultra-high-definition product photography realism.</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>outputs\images\harry_0318-0249_abstract-green_Imagen4Ultra.png</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr"/>
+      <c r="J81" s="2" t="inlineStr"/>
+      <c r="K81" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>harry_0318-0249</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>healthy-harry</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>Imagen4Ultra</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>1080x1080</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>Photorealistic DSLR lifestyle photograph. A lean athletic man in his late 20s standing in a modern kitchen, reaching into an open refrigerator.
+SUBJECT:
+Athletic male, late 20s, lean natural physique — not bulky, not a bodybuilder, normal fit person.
+Wearing a fitted grey t-shirt and training shorts. Relaxed natural posture.
+Looking at what he is holding with a calm satisfied expression. NOT posing for the camera.
+Correct human anatomy — natural hands, correct number of fingers, realistic proportions.
+WHAT HE IS HOLDING:
+A round shallow PLASTIC food container, approximately 18cm wide and 6cm tall — like a takeaway bowl.
+This is a ready-to-eat meal prep container made of plastic with a removable clear plastic snap-on lid, sealed on all sides.
+NOT a thermos. NOT a steel bottle. NOT a metal container. NOT a pan. NOT cookware. NOT a jar.
+It is a round, low-profile plastic bowl with a flat clear lid — the kind used for delivered ready meals.
+He holds it flat on his palm at chest height, lid facing up.
+REFRIGERATOR:
+Open fridge in the background with the interior light on.
+Fridge shelves are STOCKED with food — vegetables, bottles of juice, produce, other meal containers.
+Not empty. Fridge looks like a well-stocked household refrigerator.
+SCENE:
+Modern minimal kitchen. White or light stone countertop. Natural morning light from window on the left.
+Background softly out of focus.
+CAMERA: Canon R5, 35mm lens, eye-level, three-quarter body shot (head to mid-thigh), f/4, ISO 400, 5600K.
+Soft diffused natural light. Minimal shadows. True-to-life color, no filters.
+Ultra-high-definition photorealistic image, correct human anatomy, natural skin texture.</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>outputs\images\harry_0318-0249_fridge-moment_Imagen4Ultra.png</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr"/>
+      <c r="J82" s="2" t="inlineStr"/>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>harry_0318-0249</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>healthy-harry</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>Imagen4Ultra</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>1080x1080</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>Photorealistic DSLR lifestyle photograph. A lean athletic man sitting on a wooden bench in a gym locker room, with a Delicut meal prep container placed on the bench beside him.
+SUBJECT:
+Athletic male, 28-32. Lean natural physique — toned but NOT a bodybuilder, NO exaggerated or bulging muscles.
+Normal fit person with natural shoulder width. Wearing compression shorts and a sleeveless training top.
+Sitting on bench, forearms resting on knees, slight forward lean, head slightly down.
+Post-workout calm. Not looking at camera. Natural relaxed hands, correct finger count.
+PRODUCT — MUST BE IN THE IMAGE, placed on the bench to his left, in sharp focus:
+A round shallow plastic food container — compact and low-profile, approximately 18cm diameter.
+Exterior sleeve is dark spinach-green (#043F12) printed with '/delicut' in bold white sans-serif uppercase letters.
+Topped with a clear snap-on plastic lid with a raised ridge rim. No silver rim. No metallic rim.
+A small white square adhesive label sits flat on the TOP of the lid showing meal name and nutrition info.
+This container is clearly visible and prominent in the foreground — NOT absent, NOT tiny, NOT incorrect color.
+SCENE:
+Gym locker room or gym corner. Wooden bench. Lockers or plain wall softly out of focus in background.
+Subdued post-workout atmosphere. Natural side light from a high window.
+CAMERA: Canon R5, 35mm lens, slightly below bench height, mid-shot (bench to shoulders), f/4, ISO 400, 5600K.
+Product in sharp focus, subject slightly blurred. Natural side light, soft shadows.
+True-to-life color, no filters, balanced contrast.
+Ultra-high-definition photorealistic image, correct human anatomy, natural proportions.</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>outputs\images\harry_0318-0249_post-workout-bench_Imagen4Ultra.png</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr"/>
+      <c r="J83" s="2" t="inlineStr"/>
+      <c r="K83" s="2" t="inlineStr">
         <is>
           <t>pending</t>
         </is>

</xml_diff>